<commit_message>
Make BOM decide-by / order-by dates conservative; update doc dates
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01456Cj7NjpAyM7Q3YBMcz3g
</commit_message>
<xml_diff>
--- a/docs/turret_bom.xlsx
+++ b/docs/turret_bom.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="293">
   <si>
     <t xml:space="preserve">Counter-UAS Turret - Bill of Materials (one row per part)</t>
   </si>
@@ -117,7 +117,7 @@
     <t xml:space="preserve">Oct 19 (after ECE shop check)</t>
   </si>
   <si>
-    <t xml:space="preserve">Mon Oct 19 (Digi-Key) if ECE has none</t>
+    <t xml:space="preserve">Mon Oct 19 at the latest (Digi-Key, 2-3 days); Oct 26 motor test depends on it</t>
   </si>
   <si>
     <t xml:space="preserve">Motion</t>
@@ -144,7 +144,7 @@
     <t xml:space="preserve">Decided</t>
   </si>
   <si>
-    <t xml:space="preserve">Mon Oct 19 (Amazon)</t>
+    <t xml:space="preserve">Sat Oct 17 night or Mon Oct 19 at the latest (ECE will not have these; critical path for the Oct 26 test)</t>
   </si>
   <si>
     <t xml:space="preserve">Laser</t>
@@ -168,7 +168,7 @@
     <t xml:space="preserve">5 mW = Class 3R, ABOVE the project's 1 mW rule, and unbranded with no ratings, so the real power is unknown. Wall or paper target only, never aim at people, pets or shiny surfaces, never look into it. Do not call it Class 2.</t>
   </si>
   <si>
-    <t xml:space="preserve">Mon Oct 19; check arrival ZIP</t>
+    <t xml:space="preserve">Mon Oct 19 at the latest; check arrival date at checkout (marketplace seller)</t>
   </si>
   <si>
     <t xml:space="preserve">Laser switch (transistor)</t>
@@ -183,7 +183,7 @@
     <t xml:space="preserve">Qty 2 = one spare. $1.80 each, 45,069 in stock (checked Oct 17). Replaced the $8.99 Amazon 5-pack. Probably free from the ECE shop (any small logic-level MOSFET works).</t>
   </si>
   <si>
-    <t xml:space="preserve">Mon Oct 19 (Digi-Key)</t>
+    <t xml:space="preserve">Mon Oct 19 (Digi-Key, same order as the Nucleo)</t>
   </si>
   <si>
     <t xml:space="preserve">Vision</t>
@@ -204,7 +204,7 @@
     <t xml:space="preserve">You plan to unscrew it from its stand and mount just the case. When it arrives, check MJPG 1920x1080 at 30 fps is listed (v4l2-ctl --list-formats-ext on Linux, or OBS on your laptop); return it if not. Includes a 1 m USB cable with a JST connector. Only 22 ratings, 4.0 stars (100+ bought last month). The page does not list MJPEG, cable length, size or weight: get the dimensions before finishing the camera mount in CAD. Cheaper picture quality than the $39-65 cameras. Fallbacks: Arducam IMX219 autofocus $38.99 (B09BR1RNSN), ELP IMX362 $64.99 (B0DQNP1MP9).</t>
   </si>
   <si>
-    <t xml:space="preserve">Today/Sat night for Mon Oct 19 delivery (Amazon)</t>
+    <t xml:space="preserve">Sat Oct 17 night for Mon delivery, or Mon Oct 19 at the latest (does not depend on the ECE shop)</t>
   </si>
   <si>
     <t xml:space="preserve">Power</t>
@@ -228,6 +228,9 @@
     <t xml:space="preserve">Check the plug is 5.5x2.1 mm (the title does not say). The ECE shop may have a 12 V supply you can use.</t>
   </si>
   <si>
+    <t xml:space="preserve">Mon Oct 19 at the latest</t>
+  </si>
+  <si>
     <t xml:space="preserve">Barrel jack to screw terminals</t>
   </si>
   <si>
@@ -261,7 +264,7 @@
     <t xml:space="preserve">Skip Hemlock (shipping). Buy at AutoZone/O'Reilly or ask the ECE shop. Must be regular ATC size (not Mini/Micro), 15 A or more, with thick wire. Price is a guess.</t>
   </si>
   <si>
-    <t xml:space="preserve">Mon Oct 19 (local store)</t>
+    <t xml:space="preserve">Mon Oct 19 (local store, same day)</t>
   </si>
   <si>
     <t xml:space="preserve">Fuse</t>
@@ -309,7 +312,7 @@
     <t xml:space="preserve">Oct 19 (ECE shop)</t>
   </si>
   <si>
-    <t xml:space="preserve">Only if ECE has none: by Oct 22</t>
+    <t xml:space="preserve">Only if ECE has none: by Oct 21</t>
   </si>
   <si>
     <t xml:space="preserve">Wiring</t>
@@ -351,7 +354,7 @@
     <t xml:space="preserve">Oct 19 (check the Nucleo connector)</t>
   </si>
   <si>
-    <t xml:space="preserve">Only if needed</t>
+    <t xml:space="preserve">Only if needed, by Oct 21</t>
   </si>
   <si>
     <t xml:space="preserve">Mechanical</t>
@@ -372,10 +375,10 @@
     <t xml:space="preserve">Allowance only. Finish the CAD, then list exact screw sizes and lengths before buying. You can print the structure yourself.</t>
   </si>
   <si>
-    <t xml:space="preserve">After CAD is done (~Oct 24)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~Oct 24-26, before first build</t>
+    <t xml:space="preserve">After the CAD is done (target Oct 24)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">By Oct 26 (must arrive before Nov 2)</t>
   </si>
   <si>
     <t xml:space="preserve">Test</t>
@@ -399,7 +402,7 @@
     <t xml:space="preserve">PROTOTYPE 1 TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">PCB - order by Nov 2 (ships during exam dead zone). Parts depend on your design. Prices are estimates.</t>
+    <t xml:space="preserve">PCB - target order Oct 30, hard limit Nov 1 (exams start Nov 2; it ships during the dead zone). Parts depend on your design. Prices are estimates.</t>
   </si>
   <si>
     <t xml:space="preserve">PCB</t>
@@ -420,7 +423,7 @@
     <t xml:space="preserve">Pinned. Discuss after the other open items. Not a purchase.</t>
   </si>
   <si>
-    <t xml:space="preserve">Oct 30 (PCB design)</t>
+    <t xml:space="preserve">Oct 24 (so PCB layout can start)</t>
   </si>
   <si>
     <t xml:space="preserve">PCB fabrication</t>
@@ -432,19 +435,19 @@
     <t xml:space="preserve">JLCPCB / PCBWay</t>
   </si>
   <si>
-    <t xml:space="preserve">Order by Nov 2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I will not compromise on the custom PCB: it is the hardware half of my resume line. The board is a carrier board that the Nucleo plugs into, which I chose over a bare-chip board to cut risk (no fine-pitch chip soldering, no chip start-up problems) while keeping a real PCB design with real soldering. It must be ordered by Nov 2 so it ships during the exam dead zone.</t>
+    <t xml:space="preserve">Target Oct 30; hard limit Nov 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I will not compromise on the custom PCB: it is the hardware half of my resume line. The board is a carrier board that the Nucleo plugs into, which I chose over a bare-chip board to cut risk (no fine-pitch chip soldering, no chip start-up problems) while keeping a real PCB design with real soldering. It must be ordered by Nov 1 at the latest (target Oct 30) so it ships during the exam dead zone.</t>
   </si>
   <si>
     <t xml:space="preserve">Estimate includes shipping. Get a quote when the design is done.</t>
   </si>
   <si>
-    <t xml:space="preserve">Design done Oct 30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">By Nov 2</t>
+    <t xml:space="preserve">Design finished Oct 30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target Oct 30; hard limit Nov 1 (exams start Nov 2)</t>
   </si>
   <si>
     <t xml:space="preserve">Microcontroller chip (OPTIONAL, not counted)</t>
@@ -453,7 +456,7 @@
     <t xml:space="preserve">STM32G474 (package chosen in your design), same family as the Nucleo</t>
   </si>
   <si>
-    <t xml:space="preserve">Order with the PCB.</t>
+    <t xml:space="preserve">Order Oct 30 with the PCB.</t>
   </si>
   <si>
     <t xml:space="preserve">Optional and not counted, my call. The Nucleo stays on the carrier board, so the bare chip is only needed if I later go chip-down. The price was found on a Digi-Key search result.</t>
@@ -465,7 +468,7 @@
     <t xml:space="preserve">Only if going chip-down</t>
   </si>
   <si>
-    <t xml:space="preserve">Only if going chip-down (buy 2)</t>
+    <t xml:space="preserve">Only if going chip-down (with the PCB order, buy 2)</t>
   </si>
   <si>
     <t xml:space="preserve">5 V module for the Pi - OPTION A (counted)</t>
@@ -486,10 +489,10 @@
     <t xml:space="preserve">Known-good option. Needed for the final PCB (Prototype 3). In Prototype 2 the Pi runs on its wall supply instead. Option B below is cheaper but unproven.</t>
   </si>
   <si>
-    <t xml:space="preserve">~Oct 24 (a week out); before PCB layout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">With the PCB, Nov 1-3</t>
+    <t xml:space="preserve">Oct 24 (a week out); must be settled before layout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oct 30, same time as the PCB order</t>
   </si>
   <si>
     <t xml:space="preserve">5 V module for the Pi - OPTION B (not counted)</t>
@@ -510,10 +513,10 @@
     <t xml:space="preserve">The two options for the 5 V part are A (Pololu) and B (this). $5.24 normal price, 4.8 stars from only 58 reviews. The '5 A' claim is doubtful on this type of board; test with a meter and a dummy load before connecting a Pi. Footprint differs from Option A, so pick before the PCB layout is final.</t>
   </si>
   <si>
-    <t xml:space="preserve">~Oct 24 (a week out)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">If chosen: by Oct 24 (China, 1-3 weeks)</t>
+    <t xml:space="preserve">Oct 24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If you want to TEST it before the PCB order, buy by Oct 20 (ships 1-3 weeks). Ordered later, it arrives after the PCB is already sent.</t>
   </si>
   <si>
     <t xml:space="preserve">Connectors, passives, headers</t>
@@ -534,13 +537,13 @@
     <t xml:space="preserve">Oct 30</t>
   </si>
   <si>
-    <t xml:space="preserve">Nov 1-3</t>
+    <t xml:space="preserve">Oct 30, same time as the PCB order (Digi-Key, 2-3 days)</t>
   </si>
   <si>
     <t xml:space="preserve">PCB TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">PROTOTYPE 2 - order about Nov 17 (Pi wired to motors, live tracking)</t>
+    <t xml:space="preserve">PROTOTYPE 2 - order by Nov 10 (Pi wired to motors, live tracking)</t>
   </si>
   <si>
     <t xml:space="preserve">Raspberry Pi 5 (8 GB)</t>
@@ -558,16 +561,16 @@
     <t xml:space="preserve">In stock per the page; shipping time not checked.</t>
   </si>
   <si>
-    <t xml:space="preserve">I chose the 8 GB version and said I did not want the 4 GB: the RAM cannot be upgraded later, and the extra room helps with bigger models and the semester 2 drone work. I decided NOT to buy the Pi now; it is a Prototype 2 purchase, ordered by about Nov 13. Training happens on my laptop or Colab, and the Pi only runs the finished model.</t>
+    <t xml:space="preserve">I chose the 8 GB version and said I did not want the 4 GB: the RAM cannot be upgraded later, and the extra room helps with bigger models and the semester 2 drone work. I decided NOT to buy the Pi now; it is a Prototype 2 purchase, ordered by Nov 10. Training happens on my laptop or Colab, and the Pi only runs the finished model.</t>
   </si>
   <si>
     <t xml:space="preserve">PiShop also lists $175. Adafruit lists $200. The 4 GB is $110 at CanaKit (not chosen).</t>
   </si>
   <si>
-    <t xml:space="preserve">Pi + camera timing: see open question</t>
-  </si>
-  <si>
-    <t xml:space="preserve">By Nov 13 (arrive before Nov 20) unless pulled forward</t>
+    <t xml:space="preserve">Nov 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">By Nov 10 (arrive before Nov 20)</t>
   </si>
   <si>
     <t xml:space="preserve">Pi power supply</t>
@@ -582,10 +585,7 @@
     <t xml:space="preserve">Official Pi 27 W supply is $22.91 on Amazon if you want the safest option. Check reviews for 5 A output.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nov 10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">By Nov 13</t>
+    <t xml:space="preserve">By Nov 10, same CanaKit order</t>
   </si>
   <si>
     <t xml:space="preserve">Pi cooler</t>
@@ -618,7 +618,10 @@
     <t xml:space="preserve">Qty 0 so it is not counted. Prices for the same product vary by seller ($108.99 to $199.99 on Amazon; this $135.00 listing is the one you picked). Newark lists it at $89.35 (https://www.newark.com/coral/g950-01456-01/usb-accelerator-raspberry-pi/dp/26AJ4884) but says deliveries start 1/10/2027 and the lead time is 41 weeks, so it will not arrive before Dec 12. Evidence that you may not need it: Hackster's benchmark says Pi 5 TFLite performance is roughly on par with the Coral for MobileNet SSD models, and a Pi 4 CPU manages 2-5 fps.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nov 24 (after measuring the Pi alone)</t>
+    <t xml:space="preserve">Nov 23 (after measuring the Pi alone)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nov 23, only if needed (Amazon 2-day; check the price first)</t>
   </si>
   <si>
     <t xml:space="preserve">microSD card</t>
@@ -636,7 +639,7 @@
     <t xml:space="preserve">Probably free from the ECE shop or a card you already own.</t>
   </si>
   <si>
-    <t xml:space="preserve">By Nov 13 (or ECE shop)</t>
+    <t xml:space="preserve">By Nov 10 (or ECE shop)</t>
   </si>
   <si>
     <t xml:space="preserve">PROTOTYPE 2 TOTAL</t>
@@ -666,10 +669,10 @@
     <t xml:space="preserve">Only needed if you build the battery pack.</t>
   </si>
   <si>
-    <t xml:space="preserve">Late November</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Only if building a battery</t>
+    <t xml:space="preserve">Nov 22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nov 24, only if building a battery</t>
   </si>
   <si>
     <t xml:space="preserve">Power switch + reverse-polarity protection</t>
@@ -702,6 +705,9 @@
     <t xml:space="preserve">Price is my estimate for a DIY pack ($40-45). Pre-made packs I found miss the current spec or lack a stated BMS.</t>
   </si>
   <si>
+    <t xml:space="preserve">Nov 24, only if building a battery (must arrive before Dec 1)</t>
+  </si>
+  <si>
     <t xml:space="preserve">ALTERNATIVE: Stepper motor (pan + tilt)</t>
   </si>
   <si>
@@ -786,13 +792,13 @@
     <t xml:space="preserve">Closed-loop kits, dev board, laser, power parts.</t>
   </si>
   <si>
-    <t xml:space="preserve">PCB (order by Nov 2)</t>
+    <t xml:space="preserve">PCB (order target Oct 30, hard limit Nov 1)</t>
   </si>
   <si>
     <t xml:space="preserve">Estimates; depends on your design.</t>
   </si>
   <si>
-    <t xml:space="preserve">Prototype 2 (order ~Nov 17)</t>
+    <t xml:space="preserve">Prototype 2 (order by Nov 10)</t>
   </si>
   <si>
     <t xml:space="preserve">Pi 5 8 GB, power supply, cooler, Camera Module 3, cable.</t>
@@ -1847,7 +1853,7 @@
         <v>30</v>
       </c>
       <c r="R11" s="6" t="s">
-        <v>40</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1858,10 +1864,10 @@
         <v>61</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E12" s="7" t="n">
         <v>1</v>
@@ -1889,18 +1895,18 @@
         <v>65</v>
       </c>
       <c r="M12" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N12" s="11"/>
       <c r="O12" s="11"/>
       <c r="P12" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q12" s="6" t="s">
         <v>30</v>
       </c>
       <c r="R12" s="6" t="s">
-        <v>40</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1911,10 +1917,10 @@
         <v>61</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E13" s="7" t="n">
         <v>1</v>
@@ -1923,7 +1929,7 @@
         <v>24</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H13" s="8" t="n">
         <v>5</v>
@@ -1933,27 +1939,27 @@
         <v>5</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K13" s="10" t="s">
         <v>12</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="M13" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="N13" s="11"/>
       <c r="O13" s="11"/>
       <c r="P13" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q13" s="6" t="s">
         <v>30</v>
       </c>
       <c r="R13" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1964,10 +1970,10 @@
         <v>61</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E14" s="7" t="n">
         <v>1</v>
@@ -1976,7 +1982,7 @@
         <v>24</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H14" s="8" t="n">
         <v>6</v>
@@ -1986,27 +1992,27 @@
         <v>6</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K14" s="10" t="s">
         <v>12</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="M14" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="N14" s="11"/>
       <c r="O14" s="11"/>
       <c r="P14" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="Q14" s="6" t="s">
         <v>30</v>
       </c>
       <c r="R14" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2017,10 +2023,10 @@
         <v>61</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E15" s="7" t="n">
         <v>1</v>
@@ -2048,12 +2054,12 @@
         <v>27</v>
       </c>
       <c r="M15" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="N15" s="11"/>
       <c r="O15" s="11"/>
       <c r="P15" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q15" s="6" t="s">
         <v>39</v>
@@ -2070,10 +2076,10 @@
         <v>61</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E16" s="7" t="n">
         <v>0</v>
@@ -2092,27 +2098,27 @@
         <v>0</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K16" s="10" t="s">
         <v>12</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="M16" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="N16" s="11"/>
       <c r="O16" s="11"/>
       <c r="P16" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Q16" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="R16" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2120,13 +2126,13 @@
         <v>12</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E17" s="7" t="n">
         <v>0</v>
@@ -2135,7 +2141,7 @@
         <v>24</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H17" s="8" t="n">
         <v>0</v>
@@ -2145,19 +2151,19 @@
         <v>0</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K17" s="6"/>
       <c r="L17" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M17" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="N17" s="11"/>
       <c r="O17" s="11"/>
       <c r="P17" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="Q17" s="6"/>
       <c r="R17" s="6"/>
@@ -2167,13 +2173,13 @@
         <v>13</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E18" s="7" t="n">
         <v>0</v>
@@ -2182,7 +2188,7 @@
         <v>24</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H18" s="8"/>
       <c r="I18" s="9" t="str">
@@ -2190,25 +2196,25 @@
         <v/>
       </c>
       <c r="J18" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K18" s="6"/>
       <c r="L18" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M18" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="N18" s="11"/>
       <c r="O18" s="11"/>
       <c r="P18" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="Q18" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="R18" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2216,13 +2222,13 @@
         <v>14</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E19" s="7" t="n">
         <v>1</v>
@@ -2231,7 +2237,7 @@
         <v>24</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H19" s="8" t="n">
         <v>15</v>
@@ -2241,25 +2247,25 @@
         <v>15</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K19" s="6"/>
       <c r="L19" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M19" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="N19" s="11"/>
       <c r="O19" s="11"/>
       <c r="P19" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="Q19" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="R19" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2267,13 +2273,13 @@
         <v>15</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E20" s="7" t="n">
         <v>0</v>
@@ -2282,7 +2288,7 @@
         <v>24</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H20" s="8" t="n">
         <v>0</v>
@@ -2292,19 +2298,19 @@
         <v>0</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K20" s="6"/>
       <c r="L20" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M20" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N20" s="11"/>
       <c r="O20" s="11"/>
       <c r="P20" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="Q20" s="6"/>
       <c r="R20" s="6"/>
@@ -2313,7 +2319,7 @@
       <c r="A21" s="12"/>
       <c r="B21" s="12"/>
       <c r="C21" s="13" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D21" s="12"/>
       <c r="E21" s="12"/>
@@ -2336,7 +2342,7 @@
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
@@ -2361,22 +2367,22 @@
         <v>16</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E23" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H23" s="8"/>
       <c r="I23" s="9" t="str">
@@ -2384,25 +2390,25 @@
         <v/>
       </c>
       <c r="J23" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K23" s="6"/>
       <c r="L23" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M23" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="N23" s="11"/>
       <c r="O23" s="11"/>
       <c r="P23" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="Q23" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="R23" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2410,22 +2416,22 @@
         <v>17</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E24" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H24" s="8" t="n">
         <v>25</v>
@@ -2435,25 +2441,25 @@
         <v>25</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="K24" s="6"/>
       <c r="L24" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="M24" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="N24" s="11"/>
       <c r="O24" s="11"/>
       <c r="P24" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q24" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="R24" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2461,19 +2467,19 @@
         <v>18</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E25" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G25" s="5" t="s">
         <v>64</v>
@@ -2492,21 +2498,21 @@
         <v>12</v>
       </c>
       <c r="L25" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="M25" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="N25" s="11"/>
       <c r="O25" s="11"/>
       <c r="P25" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="Q25" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="R25" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2514,19 +2520,19 @@
         <v>19</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E26" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G26" s="5" t="s">
         <v>25</v>
@@ -2539,27 +2545,27 @@
         <v>32.95</v>
       </c>
       <c r="J26" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K26" s="10" t="s">
         <v>12</v>
       </c>
       <c r="L26" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="M26" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="N26" s="11"/>
       <c r="O26" s="11"/>
       <c r="P26" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="Q26" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R26" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2567,19 +2573,19 @@
         <v>20</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E27" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G27" s="5" t="s">
         <v>64</v>
@@ -2592,27 +2598,27 @@
         <v>0</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K27" s="10" t="s">
         <v>12</v>
       </c>
       <c r="L27" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="M27" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="N27" s="11"/>
       <c r="O27" s="11"/>
       <c r="P27" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="Q27" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="R27" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2620,22 +2626,22 @@
         <v>21</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E28" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H28" s="8" t="n">
         <v>15</v>
@@ -2645,32 +2651,32 @@
         <v>15</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K28" s="6"/>
       <c r="L28" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="M28" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="N28" s="11"/>
       <c r="O28" s="11"/>
       <c r="P28" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="Q28" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="R28" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12"/>
       <c r="B29" s="12"/>
       <c r="C29" s="13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D29" s="12"/>
       <c r="E29" s="12"/>
@@ -2693,7 +2699,7 @@
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -2721,16 +2727,16 @@
         <v>54</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E31" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G31" s="5" t="s">
         <v>25</v>
@@ -2743,27 +2749,27 @@
         <v>175</v>
       </c>
       <c r="J31" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K31" s="10" t="s">
         <v>12</v>
       </c>
       <c r="L31" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="M31" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="N31" s="11"/>
       <c r="O31" s="11"/>
       <c r="P31" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="Q31" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="R31" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2774,16 +2780,16 @@
         <v>54</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G32" s="5" t="s">
         <v>64</v>
@@ -2805,15 +2811,15 @@
         <v>65</v>
       </c>
       <c r="M32" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="N32" s="11"/>
       <c r="O32" s="11"/>
       <c r="P32" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="Q32" s="6" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="R32" s="6" t="s">
         <v>187</v>
@@ -2836,7 +2842,7 @@
         <v>1</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G33" s="5" t="s">
         <v>25</v>
@@ -2849,7 +2855,7 @@
         <v>11.95</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K33" s="10" t="s">
         <v>12</v>
@@ -2866,7 +2872,7 @@
         <v>192</v>
       </c>
       <c r="Q33" s="6" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="R33" s="6" t="s">
         <v>187</v>
@@ -2889,7 +2895,7 @@
         <v>0</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G34" s="5" t="s">
         <v>64</v>
@@ -2922,7 +2928,7 @@
         <v>198</v>
       </c>
       <c r="R34" s="6" t="s">
-        <v>109</v>
+        <v>199</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2933,19 +2939,19 @@
         <v>54</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E35" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H35" s="8"/>
       <c r="I35" s="9" t="str">
@@ -2953,30 +2959,30 @@
         <v/>
       </c>
       <c r="J35" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="K35" s="6"/>
       <c r="L35" s="6"/>
       <c r="M35" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="N35" s="11"/>
       <c r="O35" s="11"/>
       <c r="P35" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="Q35" s="6" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="R35" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="12"/>
       <c r="B36" s="12"/>
       <c r="C36" s="13" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="12"/>
@@ -2999,7 +3005,7 @@
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
@@ -3027,16 +3033,16 @@
         <v>61</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E38" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G38" s="5" t="s">
         <v>64</v>
@@ -3049,27 +3055,27 @@
         <v>0</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K38" s="10" t="s">
         <v>12</v>
       </c>
       <c r="L38" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="M38" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="N38" s="11"/>
       <c r="O38" s="11"/>
       <c r="P38" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="Q38" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="R38" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3080,16 +3086,16 @@
         <v>61</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G39" s="5" t="s">
         <v>25</v>
@@ -3102,27 +3108,27 @@
         <v>0</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K39" s="10" t="s">
         <v>12</v>
       </c>
       <c r="L39" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="M39" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="N39" s="11"/>
       <c r="O39" s="11"/>
       <c r="P39" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="Q39" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="R39" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3133,19 +3139,19 @@
         <v>61</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E40" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H40" s="8" t="n">
         <v>42</v>
@@ -3155,23 +3161,23 @@
         <v>0</v>
       </c>
       <c r="J40" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K40" s="6"/>
       <c r="L40" s="6"/>
       <c r="M40" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="N40" s="11"/>
       <c r="O40" s="11"/>
       <c r="P40" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="Q40" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="R40" s="6" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3182,16 +3188,16 @@
         <v>32</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="E41" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="G41" s="5" t="s">
         <v>25</v>
@@ -3210,21 +3216,21 @@
         <v>12</v>
       </c>
       <c r="L41" s="6" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="M41" s="6" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="N41" s="11"/>
       <c r="O41" s="11"/>
       <c r="P41" s="6" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="Q41" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="R41" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3235,16 +3241,16 @@
         <v>32</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E42" s="7" t="n">
         <v>0</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="G42" s="5" t="s">
         <v>64</v>
@@ -3263,26 +3269,26 @@
         <v>12</v>
       </c>
       <c r="L42" s="6" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="M42" s="6" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="N42" s="11"/>
       <c r="O42" s="11"/>
       <c r="P42" s="6" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="Q42" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="R42" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -3307,22 +3313,22 @@
         <v>32</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="E44" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H44" s="8" t="n">
         <v>50</v>
@@ -3332,25 +3338,25 @@
         <v>50</v>
       </c>
       <c r="J44" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K44" s="6"/>
       <c r="L44" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M44" s="6" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="N44" s="11"/>
       <c r="O44" s="11"/>
       <c r="P44" s="6" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="Q44" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="R44" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3358,22 +3364,22 @@
         <v>33</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E45" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H45" s="8" t="n">
         <v>30</v>
@@ -3383,32 +3389,32 @@
         <v>30</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K45" s="6"/>
       <c r="L45" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M45" s="6" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="N45" s="11"/>
       <c r="O45" s="11"/>
       <c r="P45" s="6" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="Q45" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="R45" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="12"/>
       <c r="B46" s="12"/>
       <c r="C46" s="13" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D46" s="12"/>
       <c r="E46" s="12"/>
@@ -3433,7 +3439,7 @@
       <c r="A47" s="15"/>
       <c r="B47" s="15"/>
       <c r="C47" s="16" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="D47" s="15"/>
       <c r="E47" s="15"/>
@@ -3511,83 +3517,83 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B3" s="18" t="n">
         <v>380</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B5" s="21" t="n">
         <f aca="false">SUMIFS(BOM!$I$5:$I$47,BOM!$F$5:$F$47,"P1")</f>
         <v>177.28</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B6" s="21" t="n">
         <f aca="false">SUMIFS(BOM!$I$5:$I$47,BOM!$F$5:$F$47,"PCB")</f>
         <v>72.95</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">SUMIFS(BOM!$I$5:$I$47,BOM!$F$5:$F$47,"P2")</f>
         <v>199.29</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B8" s="21" t="n">
         <f aca="false">SUMIFS(BOM!$I$5:$I$47,BOM!$F$5:$F$47,"SHIP")</f>
         <v>80</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B9" s="21" t="n">
         <f aca="false">SUMIFS(BOM!$I$5:$I$47,BOM!$F$5:$F$47,"P3")</f>
         <v>0</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B10" s="23" t="n">
         <f aca="false">SUM(B5:B9)</f>
@@ -3596,26 +3602,26 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B11" s="24" t="n">
         <f aca="false">B3-B10</f>
         <v>-149.52</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B13" s="21" t="n">
         <f aca="false">SUMIFS(BOM!$H$5:$H$47,BOM!$F$5:$F$47,"P3")</f>
         <v>57.94</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3627,75 +3633,75 @@
         <v>135</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="22" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B16" s="23" t="n">
         <f aca="false">B10</f>
         <v>529.52</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="22" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B17" s="23" t="n">
         <f aca="false">B10+B13+B14</f>
         <v>722.46</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B19" s="20" t="n">
         <f aca="false">COUNTIFS(BOM!$E$5:$E$47,"&gt;0",BOM!$G$5:$G$47,"Estimate")+COUNTIFS(BOM!$E$5:$E$47,"&gt;0",BOM!$H$5:$H$47,"")</f>
         <v>8</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B20" s="20" t="n">
         <f aca="false">COUNTIFS(BOM!$E$5:$E$47,"&gt;0",BOM!$G$5:$G$47,"Verified")</f>
         <v>8</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="22" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
   </sheetData>
@@ -3732,7 +3738,7 @@
         <v>25</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3740,47 +3746,47 @@
         <v>64</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
BOM: show local store as vendor for fuse rows on Buy Today tab
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01456Cj7NjpAyM7Q3YBMcz3g
</commit_message>
<xml_diff>
--- a/docs/turret_bom.xlsx
+++ b/docs/turret_bom.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="388">
   <si>
     <t xml:space="preserve">Counter-UAS Turret - Bill of Materials (one row per part)</t>
   </si>
@@ -1050,6 +1050,9 @@
   </si>
   <si>
     <t xml:space="preserve">Inline ATC fuse holder (regular size)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Local auto parts / hardware store</t>
   </si>
   <si>
     <t xml:space="preserve">Buy at a local auto parts store or hardware store, same day. Price is a guess. Regular ATC size, thick wire.</t>
@@ -4691,13 +4694,13 @@
         <v>5</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>94</v>
+        <v>342</v>
       </c>
       <c r="G9" s="11" t="s">
         <v>13</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4705,7 +4708,7 @@
         <v>334</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C10" s="8" t="n">
         <v>1</v>
@@ -4718,19 +4721,19 @@
         <v>6</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>94</v>
+        <v>342</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>13</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="23"/>
       <c r="B11" s="24" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C11" s="23"/>
       <c r="D11" s="23"/>
@@ -4744,7 +4747,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -4785,7 +4788,7 @@
         <v>334</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C15" s="8" t="n">
         <v>1</v>
@@ -4804,7 +4807,7 @@
         <v>13</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4812,7 +4815,7 @@
         <v>334</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C16" s="8" t="n">
         <v>1</v>
@@ -4831,13 +4834,13 @@
         <v>13</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="23"/>
       <c r="B17" s="24" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C17" s="23"/>
       <c r="D17" s="23"/>
@@ -4851,7 +4854,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -4892,7 +4895,7 @@
         <v>334</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C21" s="8" t="n">
         <v>1</v>
@@ -4909,7 +4912,7 @@
       </c>
       <c r="G21" s="7"/>
       <c r="H21" s="7" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4917,7 +4920,7 @@
         <v>334</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C22" s="8" t="n">
         <v>1</v>
@@ -4936,13 +4939,13 @@
         <v>13</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="23"/>
       <c r="B23" s="24" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C23" s="23"/>
       <c r="D23" s="23"/>
@@ -4956,7 +4959,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="2" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
   </sheetData>
@@ -5003,22 +5006,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="38" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="39" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="40" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>330</v>
@@ -5027,13 +5030,13 @@
         <v>7</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>333</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5041,16 +5044,16 @@
         <v>334</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F6" s="14"/>
     </row>
@@ -5059,16 +5062,16 @@
         <v>334</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F7" s="14"/>
     </row>
@@ -5077,13 +5080,13 @@
         <v>334</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
@@ -5093,13 +5096,13 @@
         <v>334</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E9" s="14"/>
       <c r="F9" s="14"/>
@@ -5109,16 +5112,16 @@
         <v>334</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F10" s="14"/>
     </row>
@@ -5127,23 +5130,23 @@
         <v>334</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>2</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F11" s="14"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="41"/>
       <c r="B14" s="42" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C14" s="41"/>
       <c r="D14" s="41"/>
@@ -5152,32 +5155,32 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="31" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="31" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="31" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="31" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="31" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="31" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
BOM: drop G474 Nucleo from counted cost (using the ECE shop Nucleo loan)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01456Cj7NjpAyM7Q3YBMcz3g
</commit_message>
<xml_diff>
--- a/docs/turret_bom.xlsx
+++ b/docs/turret_bom.xlsx
@@ -95,7 +95,7 @@
     <t xml:space="preserve">Control</t>
   </si>
   <si>
-    <t xml:space="preserve">Microcontroller dev board</t>
+    <t xml:space="preserve">Microcontroller dev board: NUCLEO-G474RE (OPTIONAL, not counted)</t>
   </si>
   <si>
     <t xml:space="preserve">STMicroelectronics NUCLEO-G474RE (Nucleo-64, STM32G474RE)</t>
@@ -116,13 +116,13 @@
     <t xml:space="preserve">I wanted the motor brain to be the one the industry or resume people will like better, so STM32 instead of ESP32, with one condition: it must cost only about 5 extra hours, because time is my tightest limit (10-12 hrs/week). We used Arduino-style code (PlatformIO) to hold it to that. The Nucleo-G474RE is a chip plus a built-in USB programmer on one board, so I can start testing motors right away. The G474 was chosen because the G431RB is out of stock with a 99-week lead time. Escape hatch: if no motor is turning by Oct 26, I switch to an ESP32-S3. I also chose to make my custom PCB a carrier board that this Nucleo plugs into, so this board stays in the finished turret.</t>
   </si>
   <si>
-    <t xml:space="preserve">Seen in stock (1,981) on digikey.com. Its '99 weeks' is the restock lead time, not your wait. Amazon sellers charge $88-349, do not buy there. Ask the Purdue ECE shop first; if they have a Nucleo board, skip this. 2026-10-19: the ECE shop loaned me a Nucleo-144 (row below), so I can start motor tests now. That board goes back, so the final turret still needs a Nucleo I own. This row stays counted until I decide which Nucleo the PCB is built for.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oct 24 (decide which Nucleo the PCB is built for)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oct 24 at the latest (Digi-Key). Put it in one order with the TVS so I pay shipping once.</t>
+    <t xml:space="preserve">Seen in stock (1,981) on digikey.com. Its '99 weeks' is the restock lead time, not your wait. Amazon sellers charge $88-349, do not buy there. Ask the Purdue ECE shop first; if they have a Nucleo board, skip this. 2026-10-19: the ECE shop loaned me a Nucleo-144 (row below), so I can start motor tests now. That board goes back, so if the shop wants it back before Dec 12, I buy this one. Not counted because I already have a Nucleo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only if I need my own Nucleo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only if needed (Digi-Key, 2-3 days)</t>
   </si>
   <si>
     <t xml:space="preserve">Nucleo-144 dev board (ECE shop LOAN)</t>
@@ -353,7 +353,7 @@
     <t xml:space="preserve">Use digikey.com, not the Australian site. Price/stock came from Grok, not confirmed by me (I confirmed the part and its 24.4 V clamp). If you move to 24 V later, swap this for a higher-voltage version.</t>
   </si>
   <si>
-    <t xml:space="preserve">Oct 24, in the same Digi-Key order as the Nucleo (a $0.99 part is not worth its own shipping)</t>
+    <t xml:space="preserve">Oct 30, in the same Digi-Key order as the PCB parts (a $0.99 part is not worth its own shipping)</t>
   </si>
   <si>
     <t xml:space="preserve">Bulk capacitor</t>
@@ -1067,19 +1067,13 @@
     <t xml:space="preserve">TOTAL TO BUY TODAY</t>
   </si>
   <si>
-    <t xml:space="preserve">DIGI-KEY ORDER - by Fri Oct 24 (one order, so shipping is paid once)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STMicroelectronics NUCLEO-G474RE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Needed for the final turret because the shop's Nucleo goes back. Confirm Digi-Key shows it in stock when I order.</t>
+    <t xml:space="preserve">DIGI-KEY - with the Oct 30 PCB-parts order (one order, so shipping is paid once)</t>
   </si>
   <si>
     <t xml:space="preserve">Littelfuse SMCJ15A spike protector (TVS diode)</t>
   </si>
   <si>
-    <t xml:space="preserve">A $0.99 part, so it rides in the same order as the Nucleo. The first bench power-up uses a current limit, so it can wait.</t>
+    <t xml:space="preserve">A $0.99 part, so it rides in the same Digi-Key order as the PCB parts on Oct 30. The first bench power-up uses a current limit, so it can wait.</t>
   </si>
   <si>
     <t xml:space="preserve">DIGI-KEY ORDER TOTAL (before shipping)</t>
@@ -1092,6 +1086,12 @@
   </si>
   <si>
     <t xml:space="preserve">Order by Oct 26, after the CAD is done. Must arrive before Nov 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STMicroelectronics NUCLEO-G474RE (only if the shop wants its Nucleo back)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not needed while I have the shop's loan. Only if the shop wants it back before Dec 12.</t>
   </si>
   <si>
     <t xml:space="preserve">12 V 5 A wall adapter (backup)</t>
@@ -1944,7 +1944,7 @@
       <c r="Q5" s="5"/>
       <c r="R5" s="5"/>
     </row>
-    <row r="6" customFormat="false" ht="117" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="n">
         <v>1</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>24</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>25</v>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="I6" s="10" t="n">
         <f aca="false">IF(H6="","",E6*H6)</f>
-        <v>20.13</v>
+        <v>0</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>27</v>
@@ -3040,7 +3040,7 @@
       <c r="H27" s="23"/>
       <c r="I27" s="25" t="n">
         <f aca="false">SUMIFS($I$5:$I$26,$F$5:$F$26,"P1")</f>
-        <v>154.7</v>
+        <v>134.57</v>
       </c>
       <c r="J27" s="23"/>
       <c r="K27" s="23"/>
@@ -4160,7 +4160,7 @@
       <c r="H53" s="26"/>
       <c r="I53" s="28" t="n">
         <f aca="false">I27+I35+I42+I52</f>
-        <v>506.94</v>
+        <v>486.81</v>
       </c>
       <c r="J53" s="26"/>
       <c r="K53" s="26"/>
@@ -4246,7 +4246,7 @@
       </c>
       <c r="B5" s="32" t="n">
         <f aca="false">SUMIFS(BOM!$I$5:$I$53,BOM!$F$5:$F$53,"P1")</f>
-        <v>154.7</v>
+        <v>134.57</v>
       </c>
       <c r="C5" s="31" t="s">
         <v>283</v>
@@ -4306,7 +4306,7 @@
       </c>
       <c r="B10" s="34" t="n">
         <f aca="false">SUM(B5:B9)</f>
-        <v>506.94</v>
+        <v>486.81</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4315,7 +4315,7 @@
       </c>
       <c r="B11" s="35" t="n">
         <f aca="false">B3-B10</f>
-        <v>-126.94</v>
+        <v>-106.81</v>
       </c>
       <c r="C11" s="30" t="s">
         <v>294</v>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="B16" s="34" t="n">
         <f aca="false">B10</f>
-        <v>506.94</v>
+        <v>486.81</v>
       </c>
       <c r="C16" s="30" t="s">
         <v>299</v>
@@ -4363,7 +4363,7 @@
       </c>
       <c r="B17" s="34" t="n">
         <f aca="false">B10+B13+B14</f>
-        <v>699.88</v>
+        <v>679.75</v>
       </c>
       <c r="C17" s="30" t="s">
         <v>301</v>
@@ -4387,7 +4387,7 @@
       </c>
       <c r="B20" s="31" t="n">
         <f aca="false">COUNTIFS(BOM!$E$5:$E$53,"&gt;0",BOM!$G$5:$G$53,"Verified")</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C20" s="30" t="s">
         <v>305</v>
@@ -4783,7 +4783,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
         <v>334</v>
       </c>
@@ -4794,11 +4794,11 @@
         <v>1</v>
       </c>
       <c r="D15" s="36" t="n">
-        <v>20.13</v>
+        <v>0.99</v>
       </c>
       <c r="E15" s="37" t="n">
         <f aca="false">C15*D15</f>
-        <v>20.13</v>
+        <v>0.99</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>27</v>
@@ -4810,84 +4810,82 @@
         <v>349</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="23"/>
+      <c r="B16" s="24" t="s">
+        <v>350</v>
+      </c>
+      <c r="C16" s="23"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="25" t="n">
+        <f aca="false">SUM(E15:E15)</f>
+        <v>0.99</v>
+      </c>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
+        <v>351</v>
+      </c>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="B16" s="7" t="s">
-        <v>350</v>
-      </c>
-      <c r="C16" s="8" t="n">
+      <c r="B20" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="C20" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="36" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="E16" s="37" t="n">
-        <f aca="false">C16*D16</f>
-        <v>0.99</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="23"/>
-      <c r="B17" s="24" t="s">
-        <v>352</v>
-      </c>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="25" t="n">
-        <f aca="false">SUM(E15:E16)</f>
-        <v>21.12</v>
-      </c>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="23"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
+      <c r="D20" s="36" t="n">
+        <v>15</v>
+      </c>
+      <c r="E20" s="37" t="n">
+        <f aca="false">C20*D20</f>
+        <v>15</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="G20" s="7"/>
+      <c r="H20" s="7" t="s">
         <v>353</v>
-      </c>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
-        <v>329</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>330</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>331</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>332</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G20" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H20" s="4" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4901,16 +4899,18 @@
         <v>1</v>
       </c>
       <c r="D21" s="36" t="n">
-        <v>15</v>
+        <v>20.13</v>
       </c>
       <c r="E21" s="37" t="n">
         <f aca="false">C21*D21</f>
-        <v>15</v>
+        <v>20.13</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="G21" s="7"/>
+        <v>27</v>
+      </c>
+      <c r="G21" s="11" t="s">
+        <v>13</v>
+      </c>
       <c r="H21" s="7" t="s">
         <v>355</v>
       </c>
@@ -4950,8 +4950,8 @@
       <c r="C23" s="23"/>
       <c r="D23" s="23"/>
       <c r="E23" s="25" t="n">
-        <f aca="false">SUM(E21:E22)</f>
-        <v>26.99</v>
+        <f aca="false">SUM(E20:E22)</f>
+        <v>47.12</v>
       </c>
       <c r="F23" s="23"/>
       <c r="G23" s="23"/>
@@ -4966,7 +4966,7 @@
   <mergeCells count="3">
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A18:H18"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="G6" r:id="rId1" display="Link"/>
@@ -4975,7 +4975,7 @@
     <hyperlink ref="G9" r:id="rId4" display="Link"/>
     <hyperlink ref="G10" r:id="rId5" display="Link"/>
     <hyperlink ref="G15" r:id="rId6" display="Link"/>
-    <hyperlink ref="G16" r:id="rId7" display="Link"/>
+    <hyperlink ref="G21" r:id="rId7" display="Link"/>
     <hyperlink ref="G22" r:id="rId8" display="Link"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
BOM: add S42C listing parameters (12-24 V, 1.65 A) to motor kit note
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01456Cj7NjpAyM7Q3YBMcz3g
</commit_message>
<xml_diff>
--- a/docs/turret_bom.xlsx
+++ b/docs/turret_bom.xlsx
@@ -170,7 +170,7 @@
     <t xml:space="preserve">Closed-loop motors were in the original spec: backlash and lost steps were named as a top failure risk, and a turret has to turn fast to track a moving target without losing its aim. I need motors soon so I can start the CAD, the breadboard wiring and model training, so the pick had to arrive in days. The BTT S42C kit includes the motor, the driver and the position sensor, so there is nothing to match up, costs $39.99 each, and Amazon showed delivery Oct 18. Plain steppers with separate drivers (about $50 for two axes) were rejected as open-loop. I chose 12 V for the motor rail because a 12 V battery is much cheaper than a 24 V one, and my rule was: if it is not that much slower, go 12 V. The 24 V hedge came from my worry that a turret must move fast: the PCB parts are rated for 24 V so I can upgrade later without a new board.</t>
   </si>
   <si>
-    <t xml:space="preserve">Motor is included per the listing title ('S42C V1.1 + Metal Protective Cover + Motor'). Voltage is not stated on the page; BTT's V1.0 manual rates 1.65 A at 12 V. Power it first from the bench supply at 12 V with about a 1 A current limit. Pinout in the V1.0 manual may differ from V1.1, so read the labels printed on your board. 30-day free returns if a unit is dead (some reviewers report dead units).</t>
+    <t xml:space="preserve">Motor is included per the listing title ('S42C V1.1 + Metal Protective Cover + Motor'). Listing parameters image (checked Oct 19): motor supply 12-24 V, max current 1650 mA at 12 V, no-load 620 mA at 12 V, Step/Dir input, 14-bit encoder, 2000 rpm max, STM32G031. Two motors can pull about 3.3 A together at max, so set each motor's current near 1 A on the 3 A loan adapter. Power it first at 12 V with about a 1 A current limit. Motor torque is not stated, and the V1.0 manual pinout may differ from V1.1, so read the labels printed on the board. Check the Amazon delivery address is Purdue, not Palo Alto. 30-day free returns if a unit is dead (some reviewers report dead units).</t>
   </si>
   <si>
     <t xml:space="preserve">Decided</t>
@@ -2048,7 +2048,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="168.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="n">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
BOM: switch laser to WOWOONE 5 mW 10-pack (Amazon, arrives Oct 21)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01456Cj7NjpAyM7Q3YBMcz3g
</commit_message>
<xml_diff>
--- a/docs/turret_bom.xlsx
+++ b/docs/turret_bom.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="387">
   <si>
     <t xml:space="preserve">Counter-UAS Turret - Bill of Materials (one row per part)</t>
   </si>
@@ -185,22 +185,19 @@
     <t xml:space="preserve">Laser module (lock-on indicator)</t>
   </si>
   <si>
-    <t xml:space="preserve">AREALER 4-pack 5 mW 650 nm red dot laser modules, 5 V (Walmart item 14322024651)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Walmart</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Free shipping; arrival date needs your ZIP code (not checked).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I want the laser in Prototype 1 because I want to see the result of it firing when the model detects. I chose this cheap 4-pack ($7.61) over the $25 Quarton to save about $17 and said not to worry about the maker's power guarantee. 4 modules also means spares while I test the wiring.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 mW = Class 3R, ABOVE the project's 1 mW rule, and unbranded with no ratings, so the real power is unknown. Wall or paper target only, never aim at people, pets or shiny surfaces, never look into it. Do not call it Class 2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mon Oct 19 at the latest; check arrival date at checkout (marketplace seller)</t>
+    <t xml:space="preserve">WOWOONE 10-pack 650 nm 5 mW red dot laser modules, 5 V, 6 mm brass body, pre-wired (Amazon B0GSQTBGJM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prime, free delivery Wed Oct 21 if ordered Oct 19 (Amazon showed this on the listing). Check the date at checkout.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I want the laser in Prototype 1 because I want to see the result of it firing when the model detects. I first picked a Walmart 4-pack, but it would not arrive in time, so I switched to this Amazon 10-pack ($6.69, arrives Wed Oct 21). I chose 5 mW over 1 mW because a 1 mW dot is barely visible, and the dot has to be seen in the demo. 10 modules means spares while I test the wiring.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 mW = Class 3R. Uses 5 V and about 20 mA, with a resistor built in, so no extra parts. Turn the barrel to focus the dot at the real distance. Best on a white target board in a dim room, 2-5 m away. Never aim at people, pets or shiny surfaces, never look into it. Some units in a pack are dim or poorly focused; test them all. Do not call it Class 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mon Oct 19 for Wed Oct 21 delivery</t>
   </si>
   <si>
     <t xml:space="preserve">Laser switch (transistor)</t>
@@ -1043,10 +1040,10 @@
     <t xml:space="preserve">Final camera for training and the turret. When it arrives, check MJPG 1920x1080 at 30 fps is listed (v4l2-ctl or OBS); return it if not.</t>
   </si>
   <si>
-    <t xml:space="preserve">AREALER 5 mW red laser 4-pack</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check the arrival date at checkout (marketplace seller). Never aim at people, pets or shiny surfaces.</t>
+    <t xml:space="preserve">WOWOONE 5 mW red laser 10-pack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prime, arrives Wed Oct 21. Test every unit; some are dim. Never aim at people, pets or shiny surfaces.</t>
   </si>
   <si>
     <t xml:space="preserve">Inline ATC fuse holder (regular size)</t>
@@ -2101,7 +2098,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="n">
         <v>4</v>
       </c>
@@ -2124,34 +2121,34 @@
         <v>26</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>7.61</v>
+        <v>6.69</v>
       </c>
       <c r="I9" s="10" t="n">
         <f aca="false">IF(H9="","",E9*H9)</f>
-        <v>7.61</v>
+        <v>6.69</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="K9" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L9" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="M9" s="7" t="s">
         <v>55</v>
-      </c>
-      <c r="M9" s="7" t="s">
-        <v>56</v>
       </c>
       <c r="N9" s="12"/>
       <c r="O9" s="12"/>
       <c r="P9" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Q9" s="7" t="s">
         <v>49</v>
       </c>
       <c r="R9" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2162,10 +2159,10 @@
         <v>51</v>
       </c>
       <c r="C10" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D10" s="14" t="s">
         <v>59</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>60</v>
       </c>
       <c r="E10" s="15" t="n">
         <v>2</v>
@@ -2184,25 +2181,25 @@
         <v>0</v>
       </c>
       <c r="J10" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K10" s="14"/>
       <c r="L10" s="14" t="s">
         <v>28</v>
       </c>
       <c r="M10" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="N10" s="12"/>
       <c r="O10" s="12"/>
       <c r="P10" s="14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="Q10" s="14" t="s">
         <v>40</v>
       </c>
       <c r="R10" s="14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="142.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2210,13 +2207,13 @@
         <v>6</v>
       </c>
       <c r="B11" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="D11" s="7" t="s">
         <v>66</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>67</v>
       </c>
       <c r="E11" s="8" t="n">
         <v>1</v>
@@ -2241,21 +2238,21 @@
         <v>13</v>
       </c>
       <c r="L11" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="M11" s="7" t="s">
         <v>68</v>
-      </c>
-      <c r="M11" s="7" t="s">
-        <v>69</v>
       </c>
       <c r="N11" s="12"/>
       <c r="O11" s="12"/>
       <c r="P11" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="Q11" s="7" t="s">
         <v>49</v>
       </c>
       <c r="R11" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2263,13 +2260,13 @@
         <v>7</v>
       </c>
       <c r="B12" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C12" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="D12" s="7" t="s">
         <v>73</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>74</v>
       </c>
       <c r="E12" s="8" t="n">
         <v>0</v>
@@ -2278,7 +2275,7 @@
         <v>25</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H12" s="9" t="n">
         <v>11.99</v>
@@ -2294,21 +2291,21 @@
         <v>13</v>
       </c>
       <c r="L12" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="M12" s="7" t="s">
         <v>76</v>
-      </c>
-      <c r="M12" s="7" t="s">
-        <v>77</v>
       </c>
       <c r="N12" s="12"/>
       <c r="O12" s="12"/>
       <c r="P12" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q12" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="Q12" s="7" t="s">
+      <c r="R12" s="7" t="s">
         <v>79</v>
-      </c>
-      <c r="R12" s="7" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2316,13 +2313,13 @@
         <v>8</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C13" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="D13" s="14" t="s">
         <v>81</v>
-      </c>
-      <c r="D13" s="14" t="s">
-        <v>82</v>
       </c>
       <c r="E13" s="15" t="n">
         <v>1</v>
@@ -2348,12 +2345,12 @@
         <v>37</v>
       </c>
       <c r="M13" s="14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="N13" s="12"/>
       <c r="O13" s="12"/>
       <c r="P13" s="14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="Q13" s="14" t="s">
         <v>40</v>
@@ -2367,13 +2364,13 @@
         <v>9</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C14" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="D14" s="19" t="s">
         <v>85</v>
-      </c>
-      <c r="D14" s="19" t="s">
-        <v>86</v>
       </c>
       <c r="E14" s="20" t="n">
         <v>1</v>
@@ -2382,7 +2379,7 @@
         <v>25</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H14" s="21" t="n">
         <v>0</v>
@@ -2392,25 +2389,25 @@
         <v>0</v>
       </c>
       <c r="J14" s="19" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K14" s="19"/>
       <c r="L14" s="19" t="s">
         <v>37</v>
       </c>
       <c r="M14" s="19" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="N14" s="12"/>
       <c r="O14" s="12"/>
       <c r="P14" s="19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="Q14" s="19" t="s">
         <v>40</v>
       </c>
       <c r="R14" s="19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2418,13 +2415,13 @@
         <v>10</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C15" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>91</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>92</v>
       </c>
       <c r="E15" s="8" t="n">
         <v>1</v>
@@ -2433,7 +2430,7 @@
         <v>25</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H15" s="9" t="n">
         <v>5</v>
@@ -2443,27 +2440,27 @@
         <v>5</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="K15" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L15" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="M15" s="7" t="s">
         <v>95</v>
-      </c>
-      <c r="M15" s="7" t="s">
-        <v>96</v>
       </c>
       <c r="N15" s="12"/>
       <c r="O15" s="12"/>
       <c r="P15" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="Q15" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="Q15" s="7" t="s">
+      <c r="R15" s="7" t="s">
         <v>98</v>
-      </c>
-      <c r="R15" s="7" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2471,13 +2468,13 @@
         <v>11</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C16" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>100</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="E16" s="8" t="n">
         <v>1</v>
@@ -2486,7 +2483,7 @@
         <v>25</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H16" s="9" t="n">
         <v>6</v>
@@ -2496,27 +2493,27 @@
         <v>6</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="K16" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N16" s="12"/>
       <c r="O16" s="12"/>
       <c r="P16" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="Q16" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="Q16" s="7" t="s">
-        <v>104</v>
-      </c>
       <c r="R16" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2524,13 +2521,13 @@
         <v>12</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C17" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>105</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>106</v>
       </c>
       <c r="E17" s="8" t="n">
         <v>1</v>
@@ -2539,7 +2536,7 @@
         <v>25</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H17" s="9" t="n">
         <v>0.99</v>
@@ -2558,18 +2555,18 @@
         <v>28</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="N17" s="12"/>
       <c r="O17" s="12"/>
       <c r="P17" s="7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Q17" s="7" t="s">
         <v>49</v>
       </c>
       <c r="R17" s="7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2577,13 +2574,13 @@
         <v>13</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C18" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="D18" s="19" t="s">
         <v>110</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>111</v>
       </c>
       <c r="E18" s="20" t="n">
         <v>2</v>
@@ -2592,7 +2589,7 @@
         <v>25</v>
       </c>
       <c r="G18" s="18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H18" s="21" t="n">
         <v>0</v>
@@ -2602,25 +2599,25 @@
         <v>0</v>
       </c>
       <c r="J18" s="19" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K18" s="19"/>
       <c r="L18" s="19" t="s">
         <v>37</v>
       </c>
       <c r="M18" s="19" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="N18" s="12"/>
       <c r="O18" s="12"/>
       <c r="P18" s="19" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="Q18" s="19" t="s">
         <v>40</v>
       </c>
       <c r="R18" s="19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2628,13 +2625,13 @@
         <v>14</v>
       </c>
       <c r="B19" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="C19" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="C19" s="19" t="s">
+      <c r="D19" s="19" t="s">
         <v>115</v>
-      </c>
-      <c r="D19" s="19" t="s">
-        <v>116</v>
       </c>
       <c r="E19" s="20" t="n">
         <v>1</v>
@@ -2643,7 +2640,7 @@
         <v>25</v>
       </c>
       <c r="G19" s="18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H19" s="21" t="n">
         <v>0</v>
@@ -2653,25 +2650,25 @@
         <v>0</v>
       </c>
       <c r="J19" s="19" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K19" s="19"/>
       <c r="L19" s="19" t="s">
         <v>37</v>
       </c>
       <c r="M19" s="19" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="N19" s="12"/>
       <c r="O19" s="12"/>
       <c r="P19" s="19" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="Q19" s="19" t="s">
         <v>40</v>
       </c>
       <c r="R19" s="19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2679,13 +2676,13 @@
         <v>15</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C20" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="D20" s="19" t="s">
         <v>119</v>
-      </c>
-      <c r="D20" s="19" t="s">
-        <v>120</v>
       </c>
       <c r="E20" s="20" t="n">
         <v>1</v>
@@ -2694,7 +2691,7 @@
         <v>25</v>
       </c>
       <c r="G20" s="18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H20" s="21" t="n">
         <v>0</v>
@@ -2704,25 +2701,25 @@
         <v>0</v>
       </c>
       <c r="J20" s="19" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K20" s="19"/>
       <c r="L20" s="19" t="s">
         <v>37</v>
       </c>
       <c r="M20" s="19" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="N20" s="12"/>
       <c r="O20" s="12"/>
       <c r="P20" s="19" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="Q20" s="19" t="s">
         <v>40</v>
       </c>
       <c r="R20" s="19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2730,13 +2727,13 @@
         <v>16</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C21" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="D21" s="14" t="s">
         <v>123</v>
-      </c>
-      <c r="D21" s="14" t="s">
-        <v>124</v>
       </c>
       <c r="E21" s="15" t="n">
         <v>1</v>
@@ -2762,18 +2759,18 @@
         <v>37</v>
       </c>
       <c r="M21" s="14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="N21" s="12"/>
       <c r="O21" s="12"/>
       <c r="P21" s="14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="Q21" s="14" t="s">
         <v>40</v>
       </c>
       <c r="R21" s="14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2781,13 +2778,13 @@
         <v>17</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C22" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="D22" s="19" t="s">
         <v>127</v>
-      </c>
-      <c r="D22" s="19" t="s">
-        <v>128</v>
       </c>
       <c r="E22" s="20" t="n">
         <v>1</v>
@@ -2796,7 +2793,7 @@
         <v>25</v>
       </c>
       <c r="G22" s="18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H22" s="21" t="n">
         <v>0</v>
@@ -2806,25 +2803,25 @@
         <v>0</v>
       </c>
       <c r="J22" s="19" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="K22" s="19"/>
       <c r="L22" s="19" t="s">
         <v>37</v>
       </c>
       <c r="M22" s="19" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="N22" s="12"/>
       <c r="O22" s="12"/>
       <c r="P22" s="19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="Q22" s="19" t="s">
         <v>40</v>
       </c>
       <c r="R22" s="19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2832,13 +2829,13 @@
         <v>18</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C23" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="D23" s="14" t="s">
         <v>131</v>
-      </c>
-      <c r="D23" s="14" t="s">
-        <v>132</v>
       </c>
       <c r="E23" s="15" t="n">
         <v>1</v>
@@ -2864,18 +2861,18 @@
         <v>37</v>
       </c>
       <c r="M23" s="14" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N23" s="12"/>
       <c r="O23" s="12"/>
       <c r="P23" s="14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="Q23" s="14" t="s">
         <v>40</v>
       </c>
       <c r="R23" s="14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2883,13 +2880,13 @@
         <v>19</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C24" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="D24" s="14" t="s">
         <v>135</v>
-      </c>
-      <c r="D24" s="14" t="s">
-        <v>136</v>
       </c>
       <c r="E24" s="15" t="n">
         <v>1</v>
@@ -2915,18 +2912,18 @@
         <v>37</v>
       </c>
       <c r="M24" s="14" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="N24" s="12"/>
       <c r="O24" s="12"/>
       <c r="P24" s="14" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="Q24" s="14" t="s">
         <v>40</v>
       </c>
       <c r="R24" s="14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2934,13 +2931,13 @@
         <v>20</v>
       </c>
       <c r="B25" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="C25" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="D25" s="7" t="s">
         <v>140</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>141</v>
       </c>
       <c r="E25" s="8" t="n">
         <v>1</v>
@@ -2949,7 +2946,7 @@
         <v>25</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H25" s="9" t="n">
         <v>15</v>
@@ -2959,25 +2956,25 @@
         <v>15</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K25" s="7"/>
       <c r="L25" s="7" t="s">
         <v>37</v>
       </c>
       <c r="M25" s="7" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="N25" s="12"/>
       <c r="O25" s="12"/>
       <c r="P25" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q25" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="Q25" s="7" t="s">
+      <c r="R25" s="7" t="s">
         <v>145</v>
-      </c>
-      <c r="R25" s="7" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2985,13 +2982,13 @@
         <v>21</v>
       </c>
       <c r="B26" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="C26" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="D26" s="7" t="s">
         <v>148</v>
-      </c>
-      <c r="D26" s="7" t="s">
-        <v>149</v>
       </c>
       <c r="E26" s="8" t="n">
         <v>0</v>
@@ -3000,7 +2997,7 @@
         <v>25</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H26" s="9" t="n">
         <v>0</v>
@@ -3017,12 +3014,12 @@
         <v>37</v>
       </c>
       <c r="M26" s="7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="N26" s="12"/>
       <c r="O26" s="12"/>
       <c r="P26" s="7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="Q26" s="7"/>
       <c r="R26" s="7"/>
@@ -3031,7 +3028,7 @@
       <c r="A27" s="23"/>
       <c r="B27" s="23"/>
       <c r="C27" s="24" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D27" s="23"/>
       <c r="E27" s="23"/>
@@ -3040,7 +3037,7 @@
       <c r="H27" s="23"/>
       <c r="I27" s="25" t="n">
         <f aca="false">SUMIFS($I$5:$I$26,$F$5:$F$26,"P1")</f>
-        <v>134.57</v>
+        <v>133.65</v>
       </c>
       <c r="J27" s="23"/>
       <c r="K27" s="23"/>
@@ -3054,7 +3051,7 @@
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -3079,22 +3076,22 @@
         <v>22</v>
       </c>
       <c r="B29" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="C29" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="D29" s="7" t="s">
         <v>156</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>157</v>
       </c>
       <c r="E29" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H29" s="9"/>
       <c r="I29" s="10" t="str">
@@ -3109,15 +3106,15 @@
         <v>37</v>
       </c>
       <c r="M29" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="N29" s="12"/>
       <c r="O29" s="12"/>
       <c r="P29" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="Q29" s="7" t="s">
         <v>160</v>
-      </c>
-      <c r="Q29" s="7" t="s">
-        <v>161</v>
       </c>
       <c r="R29" s="7" t="s">
         <v>37</v>
@@ -3128,22 +3125,22 @@
         <v>23</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C30" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="D30" s="7" t="s">
         <v>162</v>
-      </c>
-      <c r="D30" s="7" t="s">
-        <v>163</v>
       </c>
       <c r="E30" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H30" s="9" t="n">
         <v>25</v>
@@ -3153,25 +3150,25 @@
         <v>25</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K30" s="7"/>
       <c r="L30" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="M30" s="7" t="s">
         <v>165</v>
-      </c>
-      <c r="M30" s="7" t="s">
-        <v>166</v>
       </c>
       <c r="N30" s="12"/>
       <c r="O30" s="12"/>
       <c r="P30" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="Q30" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="Q30" s="7" t="s">
+      <c r="R30" s="7" t="s">
         <v>168</v>
-      </c>
-      <c r="R30" s="7" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3179,22 +3176,22 @@
         <v>24</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C31" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="D31" s="7" t="s">
         <v>170</v>
-      </c>
-      <c r="D31" s="7" t="s">
-        <v>171</v>
       </c>
       <c r="E31" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H31" s="9" t="n">
         <v>10.7</v>
@@ -3210,21 +3207,21 @@
         <v>13</v>
       </c>
       <c r="L31" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="M31" s="7" t="s">
         <v>172</v>
-      </c>
-      <c r="M31" s="7" t="s">
-        <v>173</v>
       </c>
       <c r="N31" s="12"/>
       <c r="O31" s="12"/>
       <c r="P31" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="Q31" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="Q31" s="7" t="s">
+      <c r="R31" s="7" t="s">
         <v>175</v>
-      </c>
-      <c r="R31" s="7" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3232,19 +3229,19 @@
         <v>25</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C32" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="D32" s="7" t="s">
         <v>177</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>178</v>
       </c>
       <c r="E32" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G32" s="6" t="s">
         <v>26</v>
@@ -3257,27 +3254,27 @@
         <v>32.95</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="K32" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L32" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="M32" s="7" t="s">
         <v>180</v>
-      </c>
-      <c r="M32" s="7" t="s">
-        <v>181</v>
       </c>
       <c r="N32" s="12"/>
       <c r="O32" s="12"/>
       <c r="P32" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="Q32" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="Q32" s="7" t="s">
+      <c r="R32" s="7" t="s">
         <v>183</v>
-      </c>
-      <c r="R32" s="7" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3285,22 +3282,22 @@
         <v>26</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C33" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="D33" s="7" t="s">
         <v>185</v>
-      </c>
-      <c r="D33" s="7" t="s">
-        <v>186</v>
       </c>
       <c r="E33" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H33" s="9" t="n">
         <v>5.24</v>
@@ -3310,27 +3307,27 @@
         <v>0</v>
       </c>
       <c r="J33" s="7" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="K33" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L33" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="M33" s="7" t="s">
         <v>188</v>
-      </c>
-      <c r="M33" s="7" t="s">
-        <v>189</v>
       </c>
       <c r="N33" s="12"/>
       <c r="O33" s="12"/>
       <c r="P33" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="Q33" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="Q33" s="7" t="s">
+      <c r="R33" s="7" t="s">
         <v>191</v>
-      </c>
-      <c r="R33" s="7" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3338,22 +3335,22 @@
         <v>27</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C34" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="D34" s="7" t="s">
         <v>193</v>
-      </c>
-      <c r="D34" s="7" t="s">
-        <v>194</v>
       </c>
       <c r="E34" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H34" s="9" t="n">
         <v>15</v>
@@ -3363,32 +3360,32 @@
         <v>15</v>
       </c>
       <c r="J34" s="7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="K34" s="7"/>
       <c r="L34" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="M34" s="7" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="N34" s="12"/>
       <c r="O34" s="12"/>
       <c r="P34" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="Q34" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="Q34" s="7" t="s">
+      <c r="R34" s="7" t="s">
         <v>198</v>
-      </c>
-      <c r="R34" s="7" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="23"/>
       <c r="B35" s="23"/>
       <c r="C35" s="24" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D35" s="23"/>
       <c r="E35" s="23"/>
@@ -3411,7 +3408,7 @@
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B36" s="5"/>
       <c r="C36" s="5"/>
@@ -3436,19 +3433,19 @@
         <v>28</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C37" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="D37" s="7" t="s">
         <v>202</v>
-      </c>
-      <c r="D37" s="7" t="s">
-        <v>203</v>
       </c>
       <c r="E37" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G37" s="6" t="s">
         <v>26</v>
@@ -3461,27 +3458,27 @@
         <v>175</v>
       </c>
       <c r="J37" s="7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="K37" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L37" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="M37" s="7" t="s">
         <v>206</v>
-      </c>
-      <c r="M37" s="7" t="s">
-        <v>207</v>
       </c>
       <c r="N37" s="12"/>
       <c r="O37" s="12"/>
       <c r="P37" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="Q37" s="7" t="s">
         <v>208</v>
       </c>
-      <c r="Q37" s="7" t="s">
+      <c r="R37" s="7" t="s">
         <v>209</v>
-      </c>
-      <c r="R37" s="7" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3489,22 +3486,22 @@
         <v>29</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C38" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="D38" s="7" t="s">
         <v>211</v>
-      </c>
-      <c r="D38" s="7" t="s">
-        <v>212</v>
       </c>
       <c r="E38" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H38" s="9" t="n">
         <v>12.34</v>
@@ -3520,21 +3517,21 @@
         <v>13</v>
       </c>
       <c r="L38" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="M38" s="7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="N38" s="12"/>
       <c r="O38" s="12"/>
       <c r="P38" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="Q38" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="R38" s="7" t="s">
         <v>214</v>
-      </c>
-      <c r="Q38" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="R38" s="7" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3542,19 +3539,19 @@
         <v>30</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C39" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="D39" s="7" t="s">
         <v>216</v>
-      </c>
-      <c r="D39" s="7" t="s">
-        <v>217</v>
       </c>
       <c r="E39" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G39" s="6" t="s">
         <v>26</v>
@@ -3567,27 +3564,27 @@
         <v>11.95</v>
       </c>
       <c r="J39" s="7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="K39" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L39" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="M39" s="7" t="s">
         <v>218</v>
-      </c>
-      <c r="M39" s="7" t="s">
-        <v>219</v>
       </c>
       <c r="N39" s="12"/>
       <c r="O39" s="12"/>
       <c r="P39" s="7" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="Q39" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="R39" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3595,22 +3592,22 @@
         <v>31</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C40" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="D40" s="7" t="s">
         <v>221</v>
-      </c>
-      <c r="D40" s="7" t="s">
-        <v>222</v>
       </c>
       <c r="E40" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H40" s="9" t="n">
         <v>135</v>
@@ -3626,21 +3623,21 @@
         <v>13</v>
       </c>
       <c r="L40" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="M40" s="7" t="s">
         <v>223</v>
-      </c>
-      <c r="M40" s="7" t="s">
-        <v>224</v>
       </c>
       <c r="N40" s="12"/>
       <c r="O40" s="12"/>
       <c r="P40" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="Q40" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="Q40" s="7" t="s">
+      <c r="R40" s="7" t="s">
         <v>226</v>
-      </c>
-      <c r="R40" s="7" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3648,22 +3645,22 @@
         <v>32</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C41" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="D41" s="7" t="s">
         <v>228</v>
-      </c>
-      <c r="D41" s="7" t="s">
-        <v>229</v>
       </c>
       <c r="E41" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H41" s="9"/>
       <c r="I41" s="10" t="str">
@@ -3671,30 +3668,30 @@
         <v/>
       </c>
       <c r="J41" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K41" s="7"/>
       <c r="L41" s="7"/>
       <c r="M41" s="7" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="N41" s="12"/>
       <c r="O41" s="12"/>
       <c r="P41" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="Q41" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="R41" s="7" t="s">
         <v>232</v>
-      </c>
-      <c r="Q41" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="R41" s="7" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="23"/>
       <c r="B42" s="23"/>
       <c r="C42" s="24" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D42" s="23"/>
       <c r="E42" s="23"/>
@@ -3717,7 +3714,7 @@
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B43" s="5"/>
       <c r="C43" s="5"/>
@@ -3742,22 +3739,22 @@
         <v>33</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C44" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="D44" s="7" t="s">
         <v>236</v>
-      </c>
-      <c r="D44" s="7" t="s">
-        <v>237</v>
       </c>
       <c r="E44" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H44" s="9" t="n">
         <v>6.99</v>
@@ -3767,27 +3764,27 @@
         <v>0</v>
       </c>
       <c r="J44" s="7" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="K44" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L44" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="M44" s="7" t="s">
         <v>240</v>
-      </c>
-      <c r="M44" s="7" t="s">
-        <v>241</v>
       </c>
       <c r="N44" s="12"/>
       <c r="O44" s="12"/>
       <c r="P44" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="Q44" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="Q44" s="7" t="s">
+      <c r="R44" s="7" t="s">
         <v>243</v>
-      </c>
-      <c r="R44" s="7" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3795,19 +3792,19 @@
         <v>34</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C45" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="D45" s="7" t="s">
         <v>245</v>
-      </c>
-      <c r="D45" s="7" t="s">
-        <v>246</v>
       </c>
       <c r="E45" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G45" s="6" t="s">
         <v>26</v>
@@ -3820,27 +3817,27 @@
         <v>0</v>
       </c>
       <c r="J45" s="7" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L45" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="M45" s="7" t="s">
         <v>247</v>
-      </c>
-      <c r="M45" s="7" t="s">
-        <v>248</v>
       </c>
       <c r="N45" s="12"/>
       <c r="O45" s="12"/>
       <c r="P45" s="7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="Q45" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="R45" s="7" t="s">
         <v>243</v>
-      </c>
-      <c r="R45" s="7" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3848,22 +3845,22 @@
         <v>35</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C46" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="D46" s="7" t="s">
         <v>250</v>
-      </c>
-      <c r="D46" s="7" t="s">
-        <v>251</v>
       </c>
       <c r="E46" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H46" s="9" t="n">
         <v>42</v>
@@ -3873,23 +3870,23 @@
         <v>0</v>
       </c>
       <c r="J46" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="K46" s="7"/>
       <c r="L46" s="7"/>
       <c r="M46" s="7" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="N46" s="12"/>
       <c r="O46" s="12"/>
       <c r="P46" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="Q46" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="R46" s="7" t="s">
         <v>254</v>
-      </c>
-      <c r="Q46" s="7" t="s">
-        <v>243</v>
-      </c>
-      <c r="R46" s="7" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3900,16 +3897,16 @@
         <v>42</v>
       </c>
       <c r="C47" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="D47" s="7" t="s">
         <v>256</v>
-      </c>
-      <c r="D47" s="7" t="s">
-        <v>257</v>
       </c>
       <c r="E47" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F47" s="6" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G47" s="6" t="s">
         <v>26</v>
@@ -3928,15 +3925,15 @@
         <v>13</v>
       </c>
       <c r="L47" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="M47" s="7" t="s">
         <v>259</v>
-      </c>
-      <c r="M47" s="7" t="s">
-        <v>260</v>
       </c>
       <c r="N47" s="12"/>
       <c r="O47" s="12"/>
       <c r="P47" s="7" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="Q47" s="7" t="s">
         <v>37</v>
@@ -3953,19 +3950,19 @@
         <v>42</v>
       </c>
       <c r="C48" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="D48" s="7" t="s">
         <v>262</v>
-      </c>
-      <c r="D48" s="7" t="s">
-        <v>263</v>
       </c>
       <c r="E48" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H48" s="9" t="n">
         <v>9.99</v>
@@ -3981,15 +3978,15 @@
         <v>13</v>
       </c>
       <c r="L48" s="7" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="M48" s="7" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="N48" s="12"/>
       <c r="O48" s="12"/>
       <c r="P48" s="7" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="Q48" s="7" t="s">
         <v>37</v>
@@ -4000,7 +3997,7 @@
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B49" s="5"/>
       <c r="C49" s="5"/>
@@ -4025,22 +4022,22 @@
         <v>38</v>
       </c>
       <c r="B50" s="7" t="s">
+        <v>266</v>
+      </c>
+      <c r="C50" s="7" t="s">
         <v>267</v>
       </c>
-      <c r="C50" s="7" t="s">
+      <c r="D50" s="7" t="s">
         <v>268</v>
-      </c>
-      <c r="D50" s="7" t="s">
-        <v>269</v>
       </c>
       <c r="E50" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H50" s="9" t="n">
         <v>50</v>
@@ -4057,12 +4054,12 @@
         <v>37</v>
       </c>
       <c r="M50" s="7" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="N50" s="12"/>
       <c r="O50" s="12"/>
       <c r="P50" s="7" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="Q50" s="7" t="s">
         <v>37</v>
@@ -4076,22 +4073,22 @@
         <v>39</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C51" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="D51" s="7" t="s">
         <v>273</v>
-      </c>
-      <c r="D51" s="7" t="s">
-        <v>274</v>
       </c>
       <c r="E51" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H51" s="9" t="n">
         <v>30</v>
@@ -4108,12 +4105,12 @@
         <v>37</v>
       </c>
       <c r="M51" s="7" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N51" s="12"/>
       <c r="O51" s="12"/>
       <c r="P51" s="7" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="Q51" s="7" t="s">
         <v>37</v>
@@ -4126,7 +4123,7 @@
       <c r="A52" s="23"/>
       <c r="B52" s="23"/>
       <c r="C52" s="24" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D52" s="23"/>
       <c r="E52" s="23"/>
@@ -4151,7 +4148,7 @@
       <c r="A53" s="26"/>
       <c r="B53" s="26"/>
       <c r="C53" s="27" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D53" s="26"/>
       <c r="E53" s="26"/>
@@ -4160,7 +4157,7 @@
       <c r="H53" s="26"/>
       <c r="I53" s="28" t="n">
         <f aca="false">I27+I35+I42+I52</f>
-        <v>486.81</v>
+        <v>485.89</v>
       </c>
       <c r="J53" s="26"/>
       <c r="K53" s="26"/>
@@ -4226,196 +4223,196 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B3" s="29" t="n">
         <v>380</v>
       </c>
       <c r="C3" s="30" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B5" s="32" t="n">
         <f aca="false">SUMIFS(BOM!$I$5:$I$53,BOM!$F$5:$F$53,"P1")</f>
-        <v>134.57</v>
+        <v>133.65</v>
       </c>
       <c r="C5" s="31" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="31" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B6" s="32" t="n">
         <f aca="false">SUMIFS(BOM!$I$5:$I$53,BOM!$F$5:$F$53,"PCB")</f>
         <v>72.95</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="31" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B7" s="32" t="n">
         <f aca="false">SUMIFS(BOM!$I$5:$I$53,BOM!$F$5:$F$53,"P2")</f>
         <v>199.29</v>
       </c>
       <c r="C7" s="31" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="31" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B8" s="32" t="n">
         <f aca="false">SUMIFS(BOM!$I$5:$I$53,BOM!$F$5:$F$53,"SHIP")</f>
         <v>80</v>
       </c>
       <c r="C8" s="31" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="31" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B9" s="32" t="n">
         <f aca="false">SUMIFS(BOM!$I$5:$I$53,BOM!$F$5:$F$53,"P3")</f>
         <v>0</v>
       </c>
       <c r="C9" s="31" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="33" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B10" s="34" t="n">
         <f aca="false">SUM(B5:B9)</f>
-        <v>486.81</v>
+        <v>485.89</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="33" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B11" s="35" t="n">
         <f aca="false">B3-B10</f>
-        <v>-106.81</v>
+        <v>-105.89</v>
       </c>
       <c r="C11" s="30" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="31" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B13" s="32" t="n">
         <f aca="false">SUMIFS(BOM!$H$5:$H$53,BOM!$F$5:$F$53,"P3")</f>
         <v>57.94</v>
       </c>
       <c r="C13" s="30" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="31" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B14" s="32" t="n">
         <f aca="false">SUMIFS(BOM!$H$5:$H$53,BOM!$C$5:$C$53,"*Coral*")</f>
         <v>135</v>
       </c>
       <c r="C14" s="30" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="33" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B16" s="34" t="n">
         <f aca="false">B10</f>
-        <v>486.81</v>
+        <v>485.89</v>
       </c>
       <c r="C16" s="30" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="33" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B17" s="34" t="n">
         <f aca="false">B10+B13+B14</f>
-        <v>679.75</v>
+        <v>678.83</v>
       </c>
       <c r="C17" s="30" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="31" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B19" s="31" t="n">
         <f aca="false">COUNTIFS(BOM!$E$5:$E$53,"&gt;0",BOM!$G$5:$G$53,"Estimate")+COUNTIFS(BOM!$E$5:$E$53,"&gt;0",BOM!$H$5:$H$53,"")</f>
         <v>8</v>
       </c>
       <c r="C19" s="30" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="31" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B20" s="31" t="n">
         <f aca="false">COUNTIFS(BOM!$E$5:$E$53,"&gt;0",BOM!$G$5:$G$53,"Verified")</f>
         <v>6</v>
       </c>
       <c r="C20" s="30" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="33" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="31" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="31" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="31" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="31" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
   </sheetData>
@@ -4452,71 +4449,71 @@
         <v>26</v>
       </c>
       <c r="B2" s="31" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="33" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="33" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="33" t="s">
+        <v>313</v>
+      </c>
+      <c r="B5" s="31" t="s">
         <v>314</v>
-      </c>
-      <c r="B5" s="31" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="33" t="s">
+        <v>315</v>
+      </c>
+      <c r="B6" s="31" t="s">
         <v>316</v>
-      </c>
-      <c r="B6" s="31" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="33" t="s">
+        <v>317</v>
+      </c>
+      <c r="B7" s="31" t="s">
         <v>318</v>
-      </c>
-      <c r="B7" s="31" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="33" t="s">
+        <v>319</v>
+      </c>
+      <c r="B8" s="31" t="s">
         <v>320</v>
-      </c>
-      <c r="B8" s="31" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="33" t="s">
+        <v>321</v>
+      </c>
+      <c r="B9" s="31" t="s">
         <v>322</v>
-      </c>
-      <c r="B9" s="31" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="33" t="s">
+        <v>323</v>
+      </c>
+      <c r="B10" s="31" t="s">
         <v>324</v>
-      </c>
-      <c r="B10" s="31" t="s">
-        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -4549,17 +4546,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -4571,19 +4568,19 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>329</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>330</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>331</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>332</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>12</v>
@@ -4592,15 +4589,15 @@
         <v>13</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>334</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>335</v>
       </c>
       <c r="C6" s="8" t="n">
         <v>2</v>
@@ -4619,15 +4616,15 @@
         <v>13</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>1</v>
@@ -4646,42 +4643,42 @@
         <v>13</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C8" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="36" t="n">
-        <v>7.61</v>
+        <v>6.69</v>
       </c>
       <c r="E8" s="37" t="n">
         <f aca="false">C8*D8</f>
-        <v>7.61</v>
+        <v>6.69</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="G8" s="11" t="s">
         <v>13</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C9" s="8" t="n">
         <v>1</v>
@@ -4694,21 +4691,21 @@
         <v>5</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="G9" s="11" t="s">
         <v>13</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C10" s="8" t="n">
         <v>1</v>
@@ -4721,25 +4718,25 @@
         <v>6</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>13</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="23"/>
       <c r="B11" s="24" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C11" s="23"/>
       <c r="D11" s="23"/>
       <c r="E11" s="25" t="n">
         <f aca="false">SUM(E6:E10)</f>
-        <v>118.58</v>
+        <v>117.66</v>
       </c>
       <c r="F11" s="23"/>
       <c r="G11" s="23"/>
@@ -4747,7 +4744,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -4759,19 +4756,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>329</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>330</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D14" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="E14" s="4" t="s">
         <v>331</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>332</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>12</v>
@@ -4780,15 +4777,15 @@
         <v>13</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C15" s="8" t="n">
         <v>1</v>
@@ -4807,13 +4804,13 @@
         <v>13</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="23"/>
       <c r="B16" s="24" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C16" s="23"/>
       <c r="D16" s="23"/>
@@ -4827,7 +4824,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -4839,19 +4836,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>329</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>330</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D19" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="E19" s="4" t="s">
         <v>331</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>332</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>12</v>
@@ -4860,15 +4857,15 @@
         <v>13</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C20" s="8" t="n">
         <v>1</v>
@@ -4881,19 +4878,19 @@
         <v>15</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G20" s="7"/>
       <c r="H20" s="7" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C21" s="8" t="n">
         <v>1</v>
@@ -4912,15 +4909,15 @@
         <v>13</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C22" s="8" t="n">
         <v>1</v>
@@ -4939,13 +4936,13 @@
         <v>13</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="23"/>
       <c r="B23" s="24" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C23" s="23"/>
       <c r="D23" s="23"/>
@@ -4959,7 +4956,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
   </sheetData>
@@ -5006,147 +5003,147 @@
   <sheetData>
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="38" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="39" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="40" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>364</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>333</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="14" t="s">
+        <v>366</v>
+      </c>
+      <c r="E6" s="14" t="s">
         <v>367</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>368</v>
       </c>
       <c r="F6" s="14"/>
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D7" s="14" t="s">
+        <v>369</v>
+      </c>
+      <c r="E7" s="14" t="s">
         <v>370</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>371</v>
       </c>
       <c r="F7" s="14"/>
     </row>
     <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E9" s="14"/>
       <c r="F9" s="14"/>
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D10" s="14" t="s">
+        <v>376</v>
+      </c>
+      <c r="E10" s="14" t="s">
         <v>377</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>378</v>
       </c>
       <c r="F10" s="14"/>
     </row>
     <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>2</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="F11" s="14"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="41"/>
       <c r="B14" s="42" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C14" s="41"/>
       <c r="D14" s="41"/>
@@ -5155,32 +5152,32 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="31" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="31" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="31" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="31" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="31" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="31" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
BOM: mark Oct 19 Amazon order as received, use real fuse holder and fuse kit listings
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01456Cj7NjpAyM7Q3YBMcz3g
</commit_message>
<xml_diff>
--- a/docs/turret_bom.xlsx
+++ b/docs/turret_bom.xlsx
@@ -24,12 +24,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="382">
   <si>
     <t xml:space="preserve">Counter-UAS Turret - Bill of Materials (one row per part)</t>
   </si>
   <si>
-    <t xml:space="preserve">Updated 2026-10-19. Status: Verified = I opened the live page and saw this price/stock. Needs check = price seen in a search result or unconfirmed detail. Estimate = my guess, no listing. Blue = typed-in input. Qty 0 = not counted in totals. Shipping and tax NOT included.</t>
+    <t xml:space="preserve">Updated 2026-10-23. Status: Verified = I opened the live page and saw this price/stock. Needs check = price seen in a search result or unconfirmed detail. Estimate = my guess, no listing. Blue = typed-in input. Qty 0 = not counted in totals. Shipping and tax NOT included.</t>
   </si>
   <si>
     <t xml:space="preserve">ORANGE rows = ECE SHOP LOANS: I must RETURN them (see the Return to ECE Shop tab).  PURPLE rows = from my 2k7 lab kit (free, mine).  Both cost $0 here.</t>
@@ -161,294 +161,273 @@
     <t xml:space="preserve">BIGTREETECH S42C V1.1 + metal cover + motor kit (Octobigtree)</t>
   </si>
   <si>
+    <t xml:space="preserve">Received</t>
+  </si>
+  <si>
     <t xml:space="preserve">Amazon</t>
   </si>
   <si>
-    <t xml:space="preserve">Listing showed delivery Sun Oct 18 on your screen.</t>
+    <t xml:space="preserve">Received Oct 23 (ordered Oct 19, Amazon, delivered to Purdue).</t>
   </si>
   <si>
     <t xml:space="preserve">Closed-loop motors were in the original spec: backlash and lost steps were named as a top failure risk, and a turret has to turn fast to track a moving target without losing its aim. I need motors soon so I can start the CAD, the breadboard wiring and model training, so the pick had to arrive in days. The BTT S42C kit includes the motor, the driver and the position sensor, so there is nothing to match up, costs $39.99 each, and Amazon showed delivery Oct 18. Plain steppers with separate drivers (about $50 for two axes) were rejected as open-loop. I chose 12 V for the motor rail because a 12 V battery is much cheaper than a 24 V one, and my rule was: if it is not that much slower, go 12 V. The 24 V hedge came from my worry that a turret must move fast: the PCB parts are rated for 24 V so I can upgrade later without a new board.</t>
   </si>
   <si>
-    <t xml:space="preserve">Motor is included per the listing title ('S42C V1.1 + Metal Protective Cover + Motor'). Listing parameters image (checked Oct 19): motor supply 12-24 V, max current 1650 mA at 12 V, no-load 620 mA at 12 V, Step/Dir input, 14-bit encoder, 2000 rpm max, STM32G031. Two motors can pull about 3.3 A together at max, so set each motor's current near 1 A on the 3 A loan adapter. Power it first at 12 V with about a 1 A current limit. Motor torque is not stated, and the V1.0 manual pinout may differ from V1.1, so read the labels printed on the board. Check the Amazon delivery address is Purdue, not Palo Alto. 30-day free returns if a unit is dead (some reviewers report dead units).</t>
+    <t xml:space="preserve">RECEIVED. Motor is included per the listing title ('S42C V1.1 + Metal Protective Cover + Motor'). Listing parameters image (checked Oct 19): motor supply 12-24 V, max current 1650 mA at 12 V, no-load 620 mA at 12 V, Step/Dir input, 14-bit encoder, 2000 rpm max, STM32G031. Two motors can pull about 3.3 A together at max, so set each motor's current near 1 A on the 3 A loan adapter. Power it first at 12 V with about a 1 A current limit. Motor torque is not stated, and the V1.0 manual pinout may differ from V1.1, so read the labels printed on the board. 30-day free returns if a unit is dead (some reviewers report dead units).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Received Oct 23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laser module (lock-on indicator)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WOWOONE 10-pack 650 nm 5 mW red dot laser modules, 5 V, 6 mm brass body, pre-wired (Amazon B0GSQTBGJM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Received Oct 23 (ordered Oct 19, Amazon).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I want the laser in Prototype 1 because I want to see the result of it firing when the model detects. I first picked a Walmart 4-pack, but it would not arrive in time, so I switched to this Amazon 10-pack ($6.69, arrives Wed Oct 21). I chose 5 mW over 1 mW because a 1 mW dot is barely visible, and the dot has to be seen in the demo. 10 modules means spares while I test the wiring.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RECEIVED. 5 mW = Class 3R. Uses 5 V and about 20 mA, with a resistor built in, so no extra parts. Turn the barrel to focus the dot at the real distance. Best on a white target board in a dim room, 2-5 m away. Never aim at people, pets or shiny surfaces, never look into it. Some units in a pack are dim or poorly focused; test them all. Do not call it Class 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laser switch (transistor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logic-level N-channel MOSFET: IRLU024N from the ECE shop (2 transistors in the bag; one is a small 3-leg TO-92 part, probably a 2N7000 or 2N2222A, so read the print). Backup: the RFD3055LE logic-level MOSFET in the 2k7 kit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ECE shop (RETURN) + 2k7 kit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An STM32 pin is too weak to power the laser by itself, so this small electronic switch lets the pin turn the laser on and off. The ECE shop gave me the part and my 2k7 kit has a second logic-level MOSFET, so I do not need to buy the $1.80 Digi-Key ones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaces the 2 x $1.80 Digi-Key order. The laser only draws about 40 mA, so any of these parts works. Ask the desk whether the shop wants small parts like this back.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not buying (free)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB camera (final camera)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arducam 1080p HDR autofocus USB camera module, 78 deg diagonal, metal body (ASIN B0FX47YSJQ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">My two reasons: (1) I want the model trained on the same camera the turret will actually use, because a different camera changes the picture quality and hurts training; (2) the camera mount in my CAD depends on the camera's exact size, so choosing the final camera now means I do not redo the CAD. I do NOT want to buy the Pi now, and the Pi camera only works on a Pi, so I needed a camera that plugs into both my laptop and the Pi later: a USB camera. I set a $27 ceiling and picked this Arducam for autofocus, a narrower 78-degree view, a 1 m cable in the box and a small metal body I can unscrew from its stand and mount in a printed holder. I accepted a cheaper picture than the $39-65 cameras and may upgrade once I am committed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RECEIVED. Next: check MJPG 1920x1080 at 30 fps is listed (v4l2-ctl --list-formats-ext or OBS); return it if not (30-day free returns). Measure the board, hole spacing and lens height for the CAD mount. Includes a 1 m USB cable with a JST connector.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 V 5 A wall adapter (BACKUP, not counted)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Facmogu 12 V 5 A, 60 W AC-DC adapter (ASIN B0711Q5B49)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Needs check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not seen. Check the listing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I asked whether the turret could run from a simple laptop charger for now and do the battery later, because the battery set was expensive and I cannot spend $300 in one month. A 12 V 5 A wall adapter is the cheap answer: 12 V is the motor voltage I picked, and 5 A (60 W) covers the estimated peak of about 87 W with some margin. The ECE shop may have one for free, so I will check Monday before buying.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not counted while I use the shop's Neewer 12 V 3 A loan. Buy this if the shop needs the Neewer back before Dec 12, or if 3 A keeps shutting off. Check the plug is 5.5x2.1 mm before ordering. Check the plug is 5.5x2.1 mm (the title does not say). The ECE shop may have a 12 V supply you can use.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nov 15 (only if the shop wants the Neewer back before the demo, or 3 A is too small)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nov 20 at the latest, only if needed (Amazon, 2 days)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 V 3 A wall adapter (ECE shop LOAN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEEWER NW-120300D2 power supply: 100-240 V AC in, 12 V DC 3.0 A out, barrel plug, UL listed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">It powers the two motors for P1. 12 V is the motor voltage I picked, and 3 A is enough while I set each motor's current to about 1 A. It is a free loan from the ECE shop, so I do not pay the $11.99 for the 5 A adapter yet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RETURN to the ECE shop. The label says output 12 V DC (the AC on the label is the wall side). 3 A is near the limit: two motors can pull about 3.3 A if both stall, so keep each motor's current setting near 1 A. Before connecting: check the plug is 5.5x2.1 mm with the center pin positive (+), and measure about 12 V DC at the plug. The first motor power-up should still use a bench supply set to 12 V with about a 1 A limit, if I can borrow one.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barrel jack to screw terminals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1 x 5.5 mm female DC power jack to screw terminal connector, from the 2k7 kit (kit part ELCONN-DCP.ST-M-03)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free: 2k7 kit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2k7 kit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lets me plug the wall adapter in and get two plain wires (+ and -) for the breadboard. My 2k7 lab kit already comes with one, so I do not need the $6.99 Amazon 20-pack.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaces the Amazon 20-pack. Check the loan adapter's plug really is 5.5 x 2.1 mm (it fits this jack if so).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuse holder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XIOGZAXI inline blade fuse holder, 2-pack, 12 AWG, 13.8 in wire, standard (regular) ATC (Amazon B0C9V2SW8K)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If something shorts, the fuse melts in a fraction of a second and cuts power before wires get hot. This holds the fuse in the power line.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RECEIVED. 2 holders in the pack, I need 1. The 2 x 30 A fuses that come with it are too big to protect the motors; use a 5 A fuse from the kit for P1. Holder is rated for 30 A, so it also works for the final turret's 15 A fuse.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AKOSN 55-piece standard ATO/ATC blade fuse assortment, 2 A to 40 A (Amazon B0DNCJRX18)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protects the wiring in a short. A 5 A fuse is enough for P1 on the 3 A loan adapter, and 15 A is the final-turret value, above my worst-case peak of about 10 A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RECEIVED. 5 A for P1, 15 A for the final turret. If a fuse blows, find out why before replacing it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spike protector (TVS diode)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Littelfuse SMCJ15A, 15 V standoff, DO-214AB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motors switching on and off create brief voltage spikes far above 12 V, and this part clamps them so they cannot hurt the drivers or the chip. It fits my 24 V upgrade hedge (I swap it for a higher-voltage version if I move to 24 V). It costs $0.99.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use digikey.com, not the Australian site. Price/stock came from Grok, not confirmed by me (I confirmed the part and its 24.4 V clamp). If you move to 24 V later, swap this for a higher-voltage version.</t>
   </si>
   <si>
     <t xml:space="preserve">Decided</t>
   </si>
   <si>
-    <t xml:space="preserve">Sat Oct 17 night or Mon Oct 19 at the latest (ECE will not have these; critical path for the Oct 26 test)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Laser</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Laser module (lock-on indicator)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WOWOONE 10-pack 650 nm 5 mW red dot laser modules, 5 V, 6 mm brass body, pre-wired (Amazon B0GSQTBGJM)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prime, free delivery Wed Oct 21 if ordered Oct 19 (Amazon showed this on the listing). Check the date at checkout.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I want the laser in Prototype 1 because I want to see the result of it firing when the model detects. I first picked a Walmart 4-pack, but it would not arrive in time, so I switched to this Amazon 10-pack ($6.69, arrives Wed Oct 21). I chose 5 mW over 1 mW because a 1 mW dot is barely visible, and the dot has to be seen in the demo. 10 modules means spares while I test the wiring.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 mW = Class 3R. Uses 5 V and about 20 mA, with a resistor built in, so no extra parts. Turn the barrel to focus the dot at the real distance. Best on a white target board in a dim room, 2-5 m away. Never aim at people, pets or shiny surfaces, never look into it. Some units in a pack are dim or poorly focused; test them all. Do not call it Class 2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mon Oct 19 for Wed Oct 21 delivery</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Laser switch (transistor)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Logic-level N-channel MOSFET: IRLU024N from the ECE shop (2 transistors in the bag; one is a small 3-leg TO-92 part, probably a 2N7000 or 2N2222A, so read the print). Backup: the RFD3055LE logic-level MOSFET in the 2k7 kit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ECE shop (RETURN) + 2k7 kit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">An STM32 pin is too weak to power the laser by itself, so this small electronic switch lets the pin turn the laser on and off. The ECE shop gave me the part and my 2k7 kit has a second logic-level MOSFET, so I do not need to buy the $1.80 Digi-Key ones.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaces the 2 x $1.80 Digi-Key order. The laser only draws about 40 mA, so any of these parts works. Ask the desk whether the shop wants small parts like this back.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not buying (free)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vision</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USB camera (final camera)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arducam 1080p HDR autofocus USB camera module, 78 deg diagonal, metal body (ASIN B0FX47YSJQ)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Page showed free delivery Mon Oct 19 (order within ~8 hours of Oct 17 evening).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">My two reasons: (1) I want the model trained on the same camera the turret will actually use, because a different camera changes the picture quality and hurts training; (2) the camera mount in my CAD depends on the camera's exact size, so choosing the final camera now means I do not redo the CAD. I do NOT want to buy the Pi now, and the Pi camera only works on a Pi, so I needed a camera that plugs into both my laptop and the Pi later: a USB camera. I set a $27 ceiling and picked this Arducam for autofocus, a narrower 78-degree view, a 1 m cable in the box and a small metal body I can unscrew from its stand and mount in a printed holder. I accepted a cheaper picture than the $39-65 cameras and may upgrade once I am committed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">You plan to unscrew it from its stand and mount just the case. When it arrives, check MJPG 1920x1080 at 30 fps is listed (v4l2-ctl --list-formats-ext on Linux, or OBS on your laptop); return it if not. Includes a 1 m USB cable with a JST connector. Only 22 ratings, 4.0 stars (100+ bought last month). The page does not list MJPEG, cable length, size or weight: get the dimensions before finishing the camera mount in CAD. Cheaper picture quality than the $39-65 cameras. Fallbacks: Arducam IMX219 autofocus $38.99 (B09BR1RNSN), ELP IMX362 $64.99 (B0DQNP1MP9).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sat Oct 17 night for Mon delivery, or Mon Oct 19 at the latest (does not depend on the ECE shop)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Power</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12 V 5 A wall adapter (BACKUP, not counted)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Facmogu 12 V 5 A, 60 W AC-DC adapter (ASIN B0711Q5B49)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Needs check</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not seen. Check the listing.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I asked whether the turret could run from a simple laptop charger for now and do the battery later, because the battery set was expensive and I cannot spend $300 in one month. A 12 V 5 A wall adapter is the cheap answer: 12 V is the motor voltage I picked, and 5 A (60 W) covers the estimated peak of about 87 W with some margin. The ECE shop may have one for free, so I will check Monday before buying.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not counted while I use the shop's Neewer 12 V 3 A loan. Buy this if the shop needs the Neewer back before Dec 12, or if 3 A keeps shutting off. Check the plug is 5.5x2.1 mm before ordering. Check the plug is 5.5x2.1 mm (the title does not say). The ECE shop may have a 12 V supply you can use.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nov 15 (only if the shop wants the Neewer back before the demo, or 3 A is too small)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nov 20 at the latest, only if needed (Amazon, 2 days)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12 V 3 A wall adapter (ECE shop LOAN)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NEEWER NW-120300D2 power supply: 100-240 V AC in, 12 V DC 3.0 A out, barrel plug, UL listed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">It powers the two motors for P1. 12 V is the motor voltage I picked, and 3 A is enough while I set each motor's current to about 1 A. It is a free loan from the ECE shop, so I do not pay the $11.99 for the 5 A adapter yet.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RETURN to the ECE shop. The label says output 12 V DC (the AC on the label is the wall side). 3 A is near the limit: two motors can pull about 3.3 A if both stall, so keep each motor's current setting near 1 A. Before connecting: check the plug is 5.5x2.1 mm with the center pin positive (+), and measure about 12 V DC at the plug. The first motor power-up should still use a bench supply set to 12 V with about a 1 A limit, if I can borrow one.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Barrel jack to screw terminals</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.1 x 5.5 mm female DC power jack to screw terminal connector, from the 2k7 kit (kit part ELCONN-DCP.ST-M-03)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Free: 2k7 kit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2k7 kit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lets me plug the wall adapter in and get two plain wires (+ and -) for the breadboard. My 2k7 lab kit already comes with one, so I do not need the $6.99 Amazon 20-pack.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaces the Amazon 20-pack. Check the loan adapter's plug really is 5.5 x 2.1 mm (it fits this jack if so).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuse holder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inline ATC (regular size) blade fuse holder, rated 15 A or more. Reference part: Bussmann #12, Hemlock SKU 580112</t>
+    <t xml:space="preserve">Oct 30, in the same Digi-Key order as the PCB parts (a $0.99 part is not worth its own shipping)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bulk capacitor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 uF 35 V electrolytic x2 from the 2k7 kit (kit part ELCAP-AE-35V-100U-05), used as a stand-in for the 1000 uF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A small water tank for electricity that smooths the motors' power gulps. The ECE shop's 1000 uF capacitors are only rated 16 V, which is too low for a 12 V rail that can spike, so I use my kit's 100 uF 35 V ones for P1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 uF is ten times smaller than my 1000 uF plan, which is fine for P1 on a current-limited supply because the S42C boards have their own capacitors. For the final turret, buy a 1000 uF 35 V capacitor (fallback: https://www.getfpv.com/black-xt60-lipo-pigtail-w-35v-1000uf-capacitor-12awg-3pcs.html, $10.99). Never use the shop's 16 V ones on the motor rail.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wiring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breadboard + jumper wires (2k7 kit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EurekaLeap 3220 tie-point solderless breadboard with 4 binding posts + 350-piece 22 AWG jumper wire set (both from the 2k7 kit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">My 2k7 lab kit comes with a big breadboard and a 350-piece jumper wire set, so I do not buy any.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The binding posts on the board are handy for the 12 V in and ground.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resistors (2k7 kit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resistor pack, 1/2 W 1%: 5 of most values, 10 each of 1, 100, 1k, 10k, 100k, 1M (includes 220 ohm and 10k ohm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The MOSFET needs a 220 ohm resistor on its gate and a 10k ohm resistor to hold it off. My kit has both, so I do not need the shop's.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kit part RES-120-00100-EH.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Male pin headers (ECE shop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standard single-row male pin header strips (from the shop's drawer 101)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For connecting the motor driver boards and jumper wires to the breadboard.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small parts. Ask the desk whether they want these back.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hand tools (2k7 kit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multi-purpose crimp / strip / cut tool (14-24 AWG), pocket 1/8 in screwdriver, banana-plug test leads, clamp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The kit's tool strips and cuts wire, so I do not borrow wire strippers. The small screwdriver fits terminal screws.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kit parts ELTOOL-WCS-YTH-5022-01, ELACC-TSCREWDRIVER-C-01, ELCAB-BNTPL-RB-36i-01.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB cable: USB-A to Micro-B (ECE shop LOAN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB data cable with a USB-A plug on one end and a Micro-B plug on the other (from my photos), black braided</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Nucleo's programming port looks like Micro-B. The shop gave me a cable that matches it, so I do not need to buy one.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RETURN to the ECE shop. Test it: plug it into the Nucleo and my laptop. If the board lights up but the laptop sees nothing new, it is charge-only. It plugs straight into my laptop's USB-A port.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB cable: USB-A to USB-C (ECE shop LOAN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB cable with a USB-A plug and a USB-C plug, black braided (from my photos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A second cable from the shop. Free, so I keep it as a spare.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RETURN to the ECE shop. My laptop has both USB-A and USB-C ports, so this is just a spare.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mechanical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screws, standoffs, fasteners</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3 screw assortment (motor mounts are M3 on NEMA 17) plus whatever your CAD needs</t>
   </si>
   <si>
     <t xml:space="preserve">Estimate</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto parts store / ECE shop (Hemlock = fallback)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same day at a local store (not checked). Hemlock fallback: in stock, 1-2 day delivery.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I asked what a fuse is and why I need it: it is a cheap part that melts on a short circuit and cuts power before wires get hot, and the holder lets me replace it. I chose to skip the online store (Hemlock) because of its shipping cost and to buy at an auto parts store or get it from the ECE shop. Must be a regular ATC size, rated 15 A or more.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skip Hemlock (shipping). Buy at AutoZone/O'Reilly or ask the ECE shop. Must be regular ATC size (not Mini/Micro), 15 A or more, with thick wire. Price is a guess.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oct 19 (after ECE shop check)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mon Oct 19 (local store, same day)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15 A regular-size ATC blade fuses, multi-pack. Reference part: Bussmann 4-pack, Hemlock SKU 573597</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same reasoning as the holder: protects the wiring in a short. 15 A is above the estimated 10 A peak so it will not blow during normal motor bursts. I will buy local or from the ECE shop to avoid shipping.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buy spares. If it blows, find out why before replacing it. For P1 on the 3 A loan adapter, a 5 A fuse is enough. 15 A is the final-turret value.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oct 19 (local store)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spike protector (TVS diode)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Littelfuse SMCJ15A, 15 V standoff, DO-214AB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Motors switching on and off create brief voltage spikes far above 12 V, and this part clamps them so they cannot hurt the drivers or the chip. It fits my 24 V upgrade hedge (I swap it for a higher-voltage version if I move to 24 V). It costs $0.99.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Use digikey.com, not the Australian site. Price/stock came from Grok, not confirmed by me (I confirmed the part and its 24.4 V clamp). If you move to 24 V later, swap this for a higher-voltage version.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oct 30, in the same Digi-Key order as the PCB parts (a $0.99 part is not worth its own shipping)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bulk capacitor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100 uF 35 V electrolytic x2 from the 2k7 kit (kit part ELCAP-AE-35V-100U-05), used as a stand-in for the 1000 uF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A small water tank for electricity that smooths the motors' power gulps. The ECE shop's 1000 uF capacitors are only rated 16 V, which is too low for a 12 V rail that can spike, so I use my kit's 100 uF 35 V ones for P1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100 uF is ten times smaller than my 1000 uF plan, which is fine for P1 on a current-limited supply because the S42C boards have their own capacitors. For the final turret, buy a 1000 uF 35 V capacitor (fallback: https://www.getfpv.com/black-xt60-lipo-pigtail-w-35v-1000uf-capacitor-12awg-3pcs.html, $10.99). Never use the shop's 16 V ones on the motor rail.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wiring</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Breadboard + jumper wires (2k7 kit)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EurekaLeap 3220 tie-point solderless breadboard with 4 binding posts + 350-piece 22 AWG jumper wire set (both from the 2k7 kit)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">My 2k7 lab kit comes with a big breadboard and a 350-piece jumper wire set, so I do not buy any.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The binding posts on the board are handy for the 12 V in and ground.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resistors (2k7 kit)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resistor pack, 1/2 W 1%: 5 of most values, 10 each of 1, 100, 1k, 10k, 100k, 1M (includes 220 ohm and 10k ohm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The MOSFET needs a 220 ohm resistor on its gate and a 10k ohm resistor to hold it off. My kit has both, so I do not need the shop's.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kit part RES-120-00100-EH.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Male pin headers (ECE shop)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Standard single-row male pin header strips (from the shop's drawer 101)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">For connecting the motor driver boards and jumper wires to the breadboard.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Small parts. Ask the desk whether they want these back.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hand tools (2k7 kit)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Multi-purpose crimp / strip / cut tool (14-24 AWG), pocket 1/8 in screwdriver, banana-plug test leads, clamp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The kit's tool strips and cuts wire, so I do not borrow wire strippers. The small screwdriver fits terminal screws.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kit parts ELTOOL-WCS-YTH-5022-01, ELACC-TSCREWDRIVER-C-01, ELCAB-BNTPL-RB-36i-01.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USB cable: USB-A to Micro-B (ECE shop LOAN)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USB data cable with a USB-A plug on one end and a Micro-B plug on the other (from my photos), black braided</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Nucleo's programming port looks like Micro-B. The shop gave me a cable that matches it, so I do not need to buy one.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RETURN to the ECE shop. Test it: plug it into the Nucleo and my laptop. If the board lights up but the laptop sees nothing new, it is charge-only. It plugs straight into my laptop's USB-A port.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USB cable: USB-A to USB-C (ECE shop LOAN)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USB cable with a USB-A plug and a USB-C plug, black braided (from my photos)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A second cable from the shop. Free, so I keep it as a spare.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RETURN to the ECE shop. My laptop has both USB-A and USB-C ports, so this is just a spare.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mechanical</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Screws, standoffs, fasteners</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M3 screw assortment (motor mounts are M3 on NEMA 17) plus whatever your CAD needs</t>
-  </si>
-  <si>
     <t xml:space="preserve">Amazon / hardware store</t>
   </si>
   <si>
@@ -938,7 +917,7 @@
     <t xml:space="preserve">Counted rows marked Verified</t>
   </si>
   <si>
-    <t xml:space="preserve">Seen on the live listing.</t>
+    <t xml:space="preserve">Seen on the live listing, or already received.</t>
   </si>
   <si>
     <t xml:space="preserve">What the ECE shop and my 2k7 kit covered</t>
@@ -959,6 +938,12 @@
     <t xml:space="preserve">I opened the live product page and saw this price and stock.</t>
   </si>
   <si>
+    <t xml:space="preserve">Received (green)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ordered and delivered. Price is what I actually paid.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Price came from a search result or a detail is unconfirmed. Check it before buying.</t>
   </si>
   <si>
@@ -1001,13 +986,13 @@
     <t xml:space="preserve">The laser is only a lock-on indicator. Never aim it at people, pets or shiny surfaces.</t>
   </si>
   <si>
-    <t xml:space="preserve">What I still have to BUY - Mon Oct 19, 2026</t>
+    <t xml:space="preserve">What I bought on Mon Oct 19, 2026 (all received Oct 23)</t>
   </si>
   <si>
     <t xml:space="preserve">Everything else for Prototype 1 is free: ECE shop loans (return them) and my 2k7 kit. Prices are from the BOM tab.</t>
   </si>
   <si>
-    <t xml:space="preserve">BUY TODAY (do not depend on the ECE shop)</t>
+    <t xml:space="preserve">ORDERED OCT 19 AND RECEIVED OCT 23 (Amazon order total was $128.02 with $8.38 tax)</t>
   </si>
   <si>
     <t xml:space="preserve">Done</t>
@@ -1025,46 +1010,46 @@
     <t xml:space="preserve">Notes</t>
   </si>
   <si>
+    <t xml:space="preserve">☑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BIGTREETECH S42C closed-loop motor + driver kit (pan + tilt)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Received. Needed for the Oct 26 motor test. The kit includes the motor. 30-day free returns.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arducam 1080p autofocus USB camera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Received. Check MJPG 1920x1080 at 30 fps is listed (v4l2-ctl or OBS); return it if not.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WOWOONE 5 mW red laser 10-pack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Received. Test every unit; some are dim. Never aim at people, pets or shiny surfaces.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XIOGZAXI inline fuse holder, 2-pack (12 AWG, regular ATC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Received. Use only 1; the second is a spare.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AKOSN 55-piece ATC fuse kit (2-40 A)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Received. 5 A for P1, 15 A for the final turret.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL (before tax)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIGI-KEY - with the Oct 30 PCB-parts order (one order, so shipping is paid once)</t>
+  </si>
+  <si>
     <t xml:space="preserve">☐</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BIGTREETECH S42C closed-loop motor + driver kit (pan + tilt)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Critical path: the Oct 26 motor test needs these. The ECE shop has no motors. The kit includes the motor. 30-day free returns.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arducam 1080p autofocus USB camera</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Final camera for training and the turret. When it arrives, check MJPG 1920x1080 at 30 fps is listed (v4l2-ctl or OBS); return it if not.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WOWOONE 5 mW red laser 10-pack</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prime, arrives Wed Oct 21. Test every unit; some are dim. Never aim at people, pets or shiny surfaces.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inline ATC fuse holder (regular size)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Local auto parts / hardware store</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buy at a local auto parts store or hardware store, same day. Price is a guess. Regular ATC size, thick wire.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ATC blade fuses (5-10 A for P1; 15 A for the final turret)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Local store, same day. Buy a multi-pack. Price is a guess.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL TO BUY TODAY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIGI-KEY - with the Oct 30 PCB-parts order (one order, so shipping is paid once)</t>
   </si>
   <si>
     <t xml:space="preserve">Littelfuse SMCJ15A spike protector (TVS diode)</t>
@@ -1342,14 +1327,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE4DFEC"/>
-        <bgColor rgb="FFD9E1F2"/>
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFE4DFEC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2EFDA"/>
-        <bgColor rgb="FFE4DFEC"/>
+        <fgColor rgb="FFE4DFEC"/>
+        <bgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -1402,7 +1387,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="49">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1495,15 +1480,39 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1567,11 +1576,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2045,110 +2054,110 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="168.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="n">
+    <row r="8" customFormat="false" ht="156" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="G8" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H8" s="9" t="n">
+      <c r="G8" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="H8" s="21" t="n">
         <v>39.99</v>
       </c>
-      <c r="I8" s="10" t="n">
+      <c r="I8" s="22" t="n">
         <f aca="false">IF(H8="","",E8*H8)</f>
         <v>79.98</v>
       </c>
-      <c r="J8" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="K8" s="11" t="s">
+      <c r="J8" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="K8" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="L8" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="M8" s="7" t="s">
+      <c r="L8" s="19" t="s">
         <v>47</v>
+      </c>
+      <c r="M8" s="19" t="s">
+        <v>48</v>
       </c>
       <c r="N8" s="12"/>
       <c r="O8" s="12"/>
-      <c r="P8" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q8" s="7" t="s">
+      <c r="P8" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="R8" s="7" t="s">
+      <c r="Q8" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="R8" s="19" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H9" s="9" t="n">
+      <c r="G9" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="H9" s="21" t="n">
         <v>6.69</v>
       </c>
-      <c r="I9" s="10" t="n">
+      <c r="I9" s="22" t="n">
         <f aca="false">IF(H9="","",E9*H9)</f>
         <v>6.69</v>
       </c>
-      <c r="J9" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="K9" s="11" t="s">
+      <c r="J9" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="K9" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="L9" s="7" t="s">
+      <c r="L9" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="M9" s="7" t="s">
+      <c r="M9" s="19" t="s">
         <v>55</v>
       </c>
       <c r="N9" s="12"/>
       <c r="O9" s="12"/>
-      <c r="P9" s="7" t="s">
+      <c r="P9" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="Q9" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="R9" s="7" t="s">
-        <v>57</v>
+      <c r="Q9" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="R9" s="19" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2159,10 +2168,10 @@
         <v>51</v>
       </c>
       <c r="C10" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" s="14" t="s">
         <v>58</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>59</v>
       </c>
       <c r="E10" s="15" t="n">
         <v>2</v>
@@ -2181,78 +2190,78 @@
         <v>0</v>
       </c>
       <c r="J10" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K10" s="14"/>
       <c r="L10" s="14" t="s">
         <v>28</v>
       </c>
       <c r="M10" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="N10" s="12"/>
       <c r="O10" s="12"/>
       <c r="P10" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="Q10" s="14" t="s">
         <v>40</v>
       </c>
       <c r="R10" s="14" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="117" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="19" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="142.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B11" s="7" t="s">
+      <c r="C11" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="D11" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="D11" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="G11" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H11" s="9" t="n">
+      <c r="G11" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="H11" s="21" t="n">
         <v>19.99</v>
       </c>
-      <c r="I11" s="10" t="n">
+      <c r="I11" s="22" t="n">
         <f aca="false">IF(H11="","",E11*H11)</f>
         <v>19.99</v>
       </c>
-      <c r="J11" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="K11" s="11" t="s">
+      <c r="J11" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="K11" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="L11" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="M11" s="7" t="s">
-        <v>68</v>
+      <c r="L11" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M11" s="19" t="s">
+        <v>66</v>
       </c>
       <c r="N11" s="12"/>
       <c r="O11" s="12"/>
-      <c r="P11" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q11" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="R11" s="7" t="s">
-        <v>70</v>
+      <c r="P11" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q11" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="R11" s="19" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2260,13 +2269,13 @@
         <v>7</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E12" s="8" t="n">
         <v>0</v>
@@ -2275,7 +2284,7 @@
         <v>25</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="H12" s="9" t="n">
         <v>11.99</v>
@@ -2285,27 +2294,27 @@
         <v>0</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K12" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="M12" s="7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="N12" s="12"/>
       <c r="O12" s="12"/>
       <c r="P12" s="7" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Q12" s="7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="R12" s="7" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="103.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2313,13 +2322,13 @@
         <v>8</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E13" s="15" t="n">
         <v>1</v>
@@ -2345,12 +2354,12 @@
         <v>37</v>
       </c>
       <c r="M13" s="14" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="N13" s="12"/>
       <c r="O13" s="12"/>
       <c r="P13" s="14" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="Q13" s="14" t="s">
         <v>40</v>
@@ -2360,160 +2369,160 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="18" t="n">
+      <c r="A14" s="24" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="19" t="s">
-        <v>71</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>84</v>
-      </c>
-      <c r="D14" s="19" t="s">
-        <v>85</v>
-      </c>
-      <c r="E14" s="20" t="n">
+      <c r="B14" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="D14" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="E14" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="18" t="s">
+      <c r="F14" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="G14" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="H14" s="21" t="n">
+      <c r="G14" s="24" t="s">
+        <v>83</v>
+      </c>
+      <c r="H14" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="I14" s="22" t="n">
+      <c r="I14" s="28" t="n">
         <f aca="false">IF(H14="","",E14*H14)</f>
         <v>0</v>
       </c>
-      <c r="J14" s="19" t="s">
-        <v>87</v>
-      </c>
-      <c r="K14" s="19"/>
-      <c r="L14" s="19" t="s">
+      <c r="J14" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="K14" s="25"/>
+      <c r="L14" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="M14" s="19" t="s">
-        <v>88</v>
+      <c r="M14" s="25" t="s">
+        <v>85</v>
       </c>
       <c r="N14" s="12"/>
       <c r="O14" s="12"/>
-      <c r="P14" s="19" t="s">
+      <c r="P14" s="25" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q14" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="R14" s="25" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="D15" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="E15" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="H15" s="21" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="I15" s="22" t="n">
+        <f aca="false">IF(H15="","",E15*H15)</f>
+        <v>5.99</v>
+      </c>
+      <c r="J15" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="K15" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="L15" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M15" s="19" t="s">
         <v>89</v>
-      </c>
-      <c r="Q14" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="R14" s="19" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="E15" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="H15" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="I15" s="10" t="n">
-        <f aca="false">IF(H15="","",E15*H15)</f>
-        <v>5</v>
-      </c>
-      <c r="J15" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="K15" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="L15" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="M15" s="7" t="s">
-        <v>95</v>
       </c>
       <c r="N15" s="12"/>
       <c r="O15" s="12"/>
-      <c r="P15" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="Q15" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="R15" s="7" t="s">
-        <v>98</v>
+      <c r="P15" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="Q15" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="R15" s="19" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="18" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="E16" s="8" t="n">
+      <c r="B16" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="D16" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="E16" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="G16" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="H16" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="I16" s="10" t="n">
+      <c r="G16" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="H16" s="21" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="I16" s="22" t="n">
         <f aca="false">IF(H16="","",E16*H16)</f>
-        <v>6</v>
-      </c>
-      <c r="J16" s="7" t="s">
+        <v>6.99</v>
+      </c>
+      <c r="J16" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="K16" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="L16" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="M16" s="19" t="s">
         <v>93</v>
-      </c>
-      <c r="K16" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="L16" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="M16" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="N16" s="12"/>
       <c r="O16" s="12"/>
-      <c r="P16" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="Q16" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="R16" s="7" t="s">
-        <v>98</v>
+      <c r="P16" s="19" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q16" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="R16" s="19" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2521,13 +2530,13 @@
         <v>12</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="E17" s="8" t="n">
         <v>1</v>
@@ -2536,7 +2545,7 @@
         <v>25</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="H17" s="9" t="n">
         <v>0.99</v>
@@ -2555,171 +2564,171 @@
         <v>28</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="N17" s="12"/>
       <c r="O17" s="12"/>
       <c r="P17" s="7" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="Q17" s="7" t="s">
-        <v>49</v>
+        <v>99</v>
       </c>
       <c r="R17" s="7" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="n">
+      <c r="A18" s="24" t="n">
         <v>13</v>
       </c>
-      <c r="B18" s="19" t="s">
-        <v>71</v>
-      </c>
-      <c r="C18" s="19" t="s">
-        <v>109</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>110</v>
-      </c>
-      <c r="E18" s="20" t="n">
+      <c r="B18" s="25" t="s">
+        <v>68</v>
+      </c>
+      <c r="C18" s="25" t="s">
+        <v>101</v>
+      </c>
+      <c r="D18" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="E18" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="F18" s="18" t="s">
+      <c r="F18" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="G18" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="H18" s="21" t="n">
+      <c r="G18" s="24" t="s">
+        <v>83</v>
+      </c>
+      <c r="H18" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="I18" s="22" t="n">
+      <c r="I18" s="28" t="n">
         <f aca="false">IF(H18="","",E18*H18)</f>
         <v>0</v>
       </c>
-      <c r="J18" s="19" t="s">
-        <v>87</v>
-      </c>
-      <c r="K18" s="19"/>
-      <c r="L18" s="19" t="s">
+      <c r="J18" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="K18" s="25"/>
+      <c r="L18" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="M18" s="19" t="s">
-        <v>111</v>
+      <c r="M18" s="25" t="s">
+        <v>103</v>
       </c>
       <c r="N18" s="12"/>
       <c r="O18" s="12"/>
-      <c r="P18" s="19" t="s">
-        <v>112</v>
-      </c>
-      <c r="Q18" s="19" t="s">
+      <c r="P18" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="Q18" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="R18" s="19" t="s">
-        <v>63</v>
+      <c r="R18" s="25" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="18" t="n">
+      <c r="A19" s="24" t="n">
         <v>14</v>
       </c>
-      <c r="B19" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>114</v>
-      </c>
-      <c r="D19" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="E19" s="20" t="n">
+      <c r="B19" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="C19" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="D19" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="E19" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="18" t="s">
+      <c r="F19" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="G19" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="H19" s="21" t="n">
+      <c r="G19" s="24" t="s">
+        <v>83</v>
+      </c>
+      <c r="H19" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="I19" s="22" t="n">
+      <c r="I19" s="28" t="n">
         <f aca="false">IF(H19="","",E19*H19)</f>
         <v>0</v>
       </c>
-      <c r="J19" s="19" t="s">
-        <v>87</v>
-      </c>
-      <c r="K19" s="19"/>
-      <c r="L19" s="19" t="s">
+      <c r="J19" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="K19" s="25"/>
+      <c r="L19" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="M19" s="19" t="s">
-        <v>116</v>
+      <c r="M19" s="25" t="s">
+        <v>108</v>
       </c>
       <c r="N19" s="12"/>
       <c r="O19" s="12"/>
-      <c r="P19" s="19" t="s">
-        <v>117</v>
-      </c>
-      <c r="Q19" s="19" t="s">
+      <c r="P19" s="25" t="s">
+        <v>109</v>
+      </c>
+      <c r="Q19" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="R19" s="19" t="s">
-        <v>63</v>
+      <c r="R19" s="25" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="18" t="n">
+      <c r="A20" s="24" t="n">
         <v>15</v>
       </c>
-      <c r="B20" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="C20" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="D20" s="19" t="s">
-        <v>119</v>
-      </c>
-      <c r="E20" s="20" t="n">
+      <c r="B20" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="D20" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="E20" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="F20" s="18" t="s">
+      <c r="F20" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="G20" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="H20" s="21" t="n">
+      <c r="G20" s="24" t="s">
+        <v>83</v>
+      </c>
+      <c r="H20" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="I20" s="22" t="n">
+      <c r="I20" s="28" t="n">
         <f aca="false">IF(H20="","",E20*H20)</f>
         <v>0</v>
       </c>
-      <c r="J20" s="19" t="s">
-        <v>87</v>
-      </c>
-      <c r="K20" s="19"/>
-      <c r="L20" s="19" t="s">
+      <c r="J20" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="K20" s="25"/>
+      <c r="L20" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="M20" s="19" t="s">
-        <v>120</v>
+      <c r="M20" s="25" t="s">
+        <v>112</v>
       </c>
       <c r="N20" s="12"/>
       <c r="O20" s="12"/>
-      <c r="P20" s="19" t="s">
-        <v>121</v>
-      </c>
-      <c r="Q20" s="19" t="s">
+      <c r="P20" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q20" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="R20" s="19" t="s">
-        <v>63</v>
+      <c r="R20" s="25" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2727,13 +2736,13 @@
         <v>16</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="E21" s="15" t="n">
         <v>1</v>
@@ -2759,69 +2768,69 @@
         <v>37</v>
       </c>
       <c r="M21" s="14" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="N21" s="12"/>
       <c r="O21" s="12"/>
       <c r="P21" s="14" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="Q21" s="14" t="s">
         <v>40</v>
       </c>
       <c r="R21" s="14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="18" t="n">
+      <c r="A22" s="24" t="n">
         <v>17</v>
       </c>
-      <c r="B22" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="C22" s="19" t="s">
-        <v>126</v>
-      </c>
-      <c r="D22" s="19" t="s">
-        <v>127</v>
-      </c>
-      <c r="E22" s="20" t="n">
+      <c r="B22" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="C22" s="25" t="s">
+        <v>118</v>
+      </c>
+      <c r="D22" s="25" t="s">
+        <v>119</v>
+      </c>
+      <c r="E22" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="F22" s="18" t="s">
+      <c r="F22" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="G22" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="H22" s="21" t="n">
+      <c r="G22" s="24" t="s">
+        <v>83</v>
+      </c>
+      <c r="H22" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="I22" s="22" t="n">
+      <c r="I22" s="28" t="n">
         <f aca="false">IF(H22="","",E22*H22)</f>
         <v>0</v>
       </c>
-      <c r="J22" s="19" t="s">
-        <v>87</v>
-      </c>
-      <c r="K22" s="19"/>
-      <c r="L22" s="19" t="s">
+      <c r="J22" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="K22" s="25"/>
+      <c r="L22" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="M22" s="19" t="s">
-        <v>128</v>
+      <c r="M22" s="25" t="s">
+        <v>120</v>
       </c>
       <c r="N22" s="12"/>
       <c r="O22" s="12"/>
-      <c r="P22" s="19" t="s">
-        <v>129</v>
-      </c>
-      <c r="Q22" s="19" t="s">
+      <c r="P22" s="25" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q22" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="R22" s="19" t="s">
-        <v>63</v>
+      <c r="R22" s="25" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2829,13 +2838,13 @@
         <v>18</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="E23" s="15" t="n">
         <v>1</v>
@@ -2861,18 +2870,18 @@
         <v>37</v>
       </c>
       <c r="M23" s="14" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="N23" s="12"/>
       <c r="O23" s="12"/>
       <c r="P23" s="14" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="Q23" s="14" t="s">
         <v>40</v>
       </c>
       <c r="R23" s="14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2880,13 +2889,13 @@
         <v>19</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="E24" s="15" t="n">
         <v>1</v>
@@ -2912,18 +2921,18 @@
         <v>37</v>
       </c>
       <c r="M24" s="14" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="N24" s="12"/>
       <c r="O24" s="12"/>
       <c r="P24" s="14" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="Q24" s="14" t="s">
         <v>40</v>
       </c>
       <c r="R24" s="14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2931,13 +2940,13 @@
         <v>20</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="E25" s="8" t="n">
         <v>1</v>
@@ -2946,7 +2955,7 @@
         <v>25</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>92</v>
+        <v>133</v>
       </c>
       <c r="H25" s="9" t="n">
         <v>15</v>
@@ -2956,25 +2965,25 @@
         <v>15</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="K25" s="7"/>
       <c r="L25" s="7" t="s">
         <v>37</v>
       </c>
       <c r="M25" s="7" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="N25" s="12"/>
       <c r="O25" s="12"/>
       <c r="P25" s="7" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="Q25" s="7" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="R25" s="7" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2982,13 +2991,13 @@
         <v>21</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="E26" s="8" t="n">
         <v>0</v>
@@ -2997,7 +3006,7 @@
         <v>25</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="H26" s="9" t="n">
         <v>0</v>
@@ -3014,44 +3023,44 @@
         <v>37</v>
       </c>
       <c r="M26" s="7" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="N26" s="12"/>
       <c r="O26" s="12"/>
       <c r="P26" s="7" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="Q26" s="7"/>
       <c r="R26" s="7"/>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="23"/>
-      <c r="B27" s="23"/>
-      <c r="C27" s="24" t="s">
-        <v>152</v>
-      </c>
-      <c r="D27" s="23"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="23"/>
-      <c r="H27" s="23"/>
-      <c r="I27" s="25" t="n">
+      <c r="A27" s="29"/>
+      <c r="B27" s="29"/>
+      <c r="C27" s="30" t="s">
+        <v>145</v>
+      </c>
+      <c r="D27" s="29"/>
+      <c r="E27" s="29"/>
+      <c r="F27" s="29"/>
+      <c r="G27" s="29"/>
+      <c r="H27" s="29"/>
+      <c r="I27" s="31" t="n">
         <f aca="false">SUMIFS($I$5:$I$26,$F$5:$F$26,"P1")</f>
-        <v>133.65</v>
-      </c>
-      <c r="J27" s="23"/>
-      <c r="K27" s="23"/>
-      <c r="L27" s="23"/>
-      <c r="M27" s="23"/>
-      <c r="N27" s="23"/>
-      <c r="O27" s="23"/>
-      <c r="P27" s="23"/>
-      <c r="Q27" s="23"/>
-      <c r="R27" s="23"/>
+        <v>135.63</v>
+      </c>
+      <c r="J27" s="29"/>
+      <c r="K27" s="29"/>
+      <c r="L27" s="29"/>
+      <c r="M27" s="29"/>
+      <c r="N27" s="29"/>
+      <c r="O27" s="29"/>
+      <c r="P27" s="29"/>
+      <c r="Q27" s="29"/>
+      <c r="R27" s="29"/>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -3076,22 +3085,22 @@
         <v>22</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="E29" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="H29" s="9"/>
       <c r="I29" s="10" t="str">
@@ -3106,15 +3115,15 @@
         <v>37</v>
       </c>
       <c r="M29" s="7" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="N29" s="12"/>
       <c r="O29" s="12"/>
       <c r="P29" s="7" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="Q29" s="7" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="R29" s="7" t="s">
         <v>37</v>
@@ -3125,22 +3134,22 @@
         <v>23</v>
       </c>
       <c r="B30" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="C30" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="C30" s="7" t="s">
-        <v>161</v>
-      </c>
       <c r="D30" s="7" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="E30" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>92</v>
+        <v>133</v>
       </c>
       <c r="H30" s="9" t="n">
         <v>25</v>
@@ -3150,25 +3159,25 @@
         <v>25</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="K30" s="7"/>
       <c r="L30" s="7" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="M30" s="7" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="N30" s="12"/>
       <c r="O30" s="12"/>
       <c r="P30" s="7" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="Q30" s="7" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="R30" s="7" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3176,22 +3185,22 @@
         <v>24</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="E31" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="G31" s="6" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="H31" s="9" t="n">
         <v>10.7</v>
@@ -3207,21 +3216,21 @@
         <v>13</v>
       </c>
       <c r="L31" s="7" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="M31" s="7" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="N31" s="12"/>
       <c r="O31" s="12"/>
       <c r="P31" s="7" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="Q31" s="7" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="R31" s="7" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3229,19 +3238,19 @@
         <v>25</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="E32" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="G32" s="6" t="s">
         <v>26</v>
@@ -3254,27 +3263,27 @@
         <v>32.95</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="K32" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L32" s="7" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="M32" s="7" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="N32" s="12"/>
       <c r="O32" s="12"/>
       <c r="P32" s="7" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="Q32" s="7" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="R32" s="7" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3282,22 +3291,22 @@
         <v>26</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="E33" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="H33" s="9" t="n">
         <v>5.24</v>
@@ -3307,27 +3316,27 @@
         <v>0</v>
       </c>
       <c r="J33" s="7" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="K33" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L33" s="7" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="M33" s="7" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="N33" s="12"/>
       <c r="O33" s="12"/>
       <c r="P33" s="7" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="Q33" s="7" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="R33" s="7" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3335,22 +3344,22 @@
         <v>27</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="E34" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>92</v>
+        <v>133</v>
       </c>
       <c r="H34" s="9" t="n">
         <v>15</v>
@@ -3360,55 +3369,55 @@
         <v>15</v>
       </c>
       <c r="J34" s="7" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="K34" s="7"/>
       <c r="L34" s="7" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="M34" s="7" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="N34" s="12"/>
       <c r="O34" s="12"/>
       <c r="P34" s="7" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="Q34" s="7" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="R34" s="7" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="23"/>
-      <c r="B35" s="23"/>
-      <c r="C35" s="24" t="s">
-        <v>199</v>
-      </c>
-      <c r="D35" s="23"/>
-      <c r="E35" s="23"/>
-      <c r="F35" s="23"/>
-      <c r="G35" s="23"/>
-      <c r="H35" s="23"/>
-      <c r="I35" s="25" t="n">
+      <c r="A35" s="29"/>
+      <c r="B35" s="29"/>
+      <c r="C35" s="30" t="s">
+        <v>192</v>
+      </c>
+      <c r="D35" s="29"/>
+      <c r="E35" s="29"/>
+      <c r="F35" s="29"/>
+      <c r="G35" s="29"/>
+      <c r="H35" s="29"/>
+      <c r="I35" s="31" t="n">
         <f aca="false">SUMIFS($I$5:$I$34,$F$5:$F$34,"PCB")</f>
         <v>72.95</v>
       </c>
-      <c r="J35" s="23"/>
-      <c r="K35" s="23"/>
-      <c r="L35" s="23"/>
-      <c r="M35" s="23"/>
-      <c r="N35" s="23"/>
-      <c r="O35" s="23"/>
-      <c r="P35" s="23"/>
-      <c r="Q35" s="23"/>
-      <c r="R35" s="23"/>
+      <c r="J35" s="29"/>
+      <c r="K35" s="29"/>
+      <c r="L35" s="29"/>
+      <c r="M35" s="29"/>
+      <c r="N35" s="29"/>
+      <c r="O35" s="29"/>
+      <c r="P35" s="29"/>
+      <c r="Q35" s="29"/>
+      <c r="R35" s="29"/>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="B36" s="5"/>
       <c r="C36" s="5"/>
@@ -3433,19 +3442,19 @@
         <v>28</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="E37" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="G37" s="6" t="s">
         <v>26</v>
@@ -3458,27 +3467,27 @@
         <v>175</v>
       </c>
       <c r="J37" s="7" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="K37" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L37" s="7" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="M37" s="7" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="N37" s="12"/>
       <c r="O37" s="12"/>
       <c r="P37" s="7" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="Q37" s="7" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="R37" s="7" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3486,22 +3495,22 @@
         <v>29</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="E38" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="H38" s="9" t="n">
         <v>12.34</v>
@@ -3511,27 +3520,27 @@
         <v>12.34</v>
       </c>
       <c r="J38" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K38" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L38" s="7" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="M38" s="7" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="N38" s="12"/>
       <c r="O38" s="12"/>
       <c r="P38" s="7" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="Q38" s="7" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="R38" s="7" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3539,19 +3548,19 @@
         <v>30</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="E39" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="G39" s="6" t="s">
         <v>26</v>
@@ -3564,27 +3573,27 @@
         <v>11.95</v>
       </c>
       <c r="J39" s="7" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="K39" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L39" s="7" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="M39" s="7" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="N39" s="12"/>
       <c r="O39" s="12"/>
       <c r="P39" s="7" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="Q39" s="7" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="R39" s="7" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="129.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3592,22 +3601,22 @@
         <v>31</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="E40" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="H40" s="9" t="n">
         <v>135</v>
@@ -3617,27 +3626,27 @@
         <v>0</v>
       </c>
       <c r="J40" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K40" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L40" s="7" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="M40" s="7" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="N40" s="12"/>
       <c r="O40" s="12"/>
       <c r="P40" s="7" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="Q40" s="7" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="R40" s="7" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3645,22 +3654,22 @@
         <v>32</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="E41" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="H41" s="9"/>
       <c r="I41" s="10" t="str">
@@ -3668,53 +3677,53 @@
         <v/>
       </c>
       <c r="J41" s="7" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="K41" s="7"/>
       <c r="L41" s="7"/>
       <c r="M41" s="7" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="N41" s="12"/>
       <c r="O41" s="12"/>
       <c r="P41" s="7" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="Q41" s="7" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="R41" s="7" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="23"/>
-      <c r="B42" s="23"/>
-      <c r="C42" s="24" t="s">
-        <v>233</v>
-      </c>
-      <c r="D42" s="23"/>
-      <c r="E42" s="23"/>
-      <c r="F42" s="23"/>
-      <c r="G42" s="23"/>
-      <c r="H42" s="23"/>
-      <c r="I42" s="25" t="n">
+      <c r="A42" s="29"/>
+      <c r="B42" s="29"/>
+      <c r="C42" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="D42" s="29"/>
+      <c r="E42" s="29"/>
+      <c r="F42" s="29"/>
+      <c r="G42" s="29"/>
+      <c r="H42" s="29"/>
+      <c r="I42" s="31" t="n">
         <f aca="false">SUMIFS($I$5:$I$41,$F$5:$F$41,"P2")</f>
         <v>199.29</v>
       </c>
-      <c r="J42" s="23"/>
-      <c r="K42" s="23"/>
-      <c r="L42" s="23"/>
-      <c r="M42" s="23"/>
-      <c r="N42" s="23"/>
-      <c r="O42" s="23"/>
-      <c r="P42" s="23"/>
-      <c r="Q42" s="23"/>
-      <c r="R42" s="23"/>
+      <c r="J42" s="29"/>
+      <c r="K42" s="29"/>
+      <c r="L42" s="29"/>
+      <c r="M42" s="29"/>
+      <c r="N42" s="29"/>
+      <c r="O42" s="29"/>
+      <c r="P42" s="29"/>
+      <c r="Q42" s="29"/>
+      <c r="R42" s="29"/>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B43" s="5"/>
       <c r="C43" s="5"/>
@@ -3739,22 +3748,22 @@
         <v>33</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="E44" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="H44" s="9" t="n">
         <v>6.99</v>
@@ -3764,27 +3773,27 @@
         <v>0</v>
       </c>
       <c r="J44" s="7" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="K44" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L44" s="7" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="M44" s="7" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="N44" s="12"/>
       <c r="O44" s="12"/>
       <c r="P44" s="7" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="Q44" s="7" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="R44" s="7" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3792,19 +3801,19 @@
         <v>34</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="E45" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="G45" s="6" t="s">
         <v>26</v>
@@ -3817,27 +3826,27 @@
         <v>0</v>
       </c>
       <c r="J45" s="7" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="K45" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L45" s="7" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="M45" s="7" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="N45" s="12"/>
       <c r="O45" s="12"/>
       <c r="P45" s="7" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="Q45" s="7" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="R45" s="7" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3845,22 +3854,22 @@
         <v>35</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="D46" s="7" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="E46" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="H46" s="9" t="n">
         <v>42</v>
@@ -3870,23 +3879,23 @@
         <v>0</v>
       </c>
       <c r="J46" s="7" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="K46" s="7"/>
       <c r="L46" s="7"/>
       <c r="M46" s="7" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="N46" s="12"/>
       <c r="O46" s="12"/>
       <c r="P46" s="7" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="Q46" s="7" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="R46" s="7" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3897,16 +3906,16 @@
         <v>42</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="E47" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F47" s="6" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="G47" s="6" t="s">
         <v>26</v>
@@ -3919,21 +3928,21 @@
         <v>0</v>
       </c>
       <c r="J47" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K47" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L47" s="7" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="M47" s="7" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="N47" s="12"/>
       <c r="O47" s="12"/>
       <c r="P47" s="7" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="Q47" s="7" t="s">
         <v>37</v>
@@ -3950,19 +3959,19 @@
         <v>42</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="E48" s="8" t="n">
         <v>0</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="H48" s="9" t="n">
         <v>9.99</v>
@@ -3972,21 +3981,21 @@
         <v>0</v>
       </c>
       <c r="J48" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K48" s="11" t="s">
         <v>13</v>
       </c>
       <c r="L48" s="7" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="M48" s="7" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="N48" s="12"/>
       <c r="O48" s="12"/>
       <c r="P48" s="7" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="Q48" s="7" t="s">
         <v>37</v>
@@ -3997,7 +4006,7 @@
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="B49" s="5"/>
       <c r="C49" s="5"/>
@@ -4022,22 +4031,22 @@
         <v>38</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="D50" s="7" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="E50" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>92</v>
+        <v>133</v>
       </c>
       <c r="H50" s="9" t="n">
         <v>50</v>
@@ -4054,12 +4063,12 @@
         <v>37</v>
       </c>
       <c r="M50" s="7" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="N50" s="12"/>
       <c r="O50" s="12"/>
       <c r="P50" s="7" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="Q50" s="7" t="s">
         <v>37</v>
@@ -4073,22 +4082,22 @@
         <v>39</v>
       </c>
       <c r="B51" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="D51" s="7" t="s">
         <v>266</v>
-      </c>
-      <c r="C51" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="D51" s="7" t="s">
-        <v>273</v>
       </c>
       <c r="E51" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>92</v>
+        <v>133</v>
       </c>
       <c r="H51" s="9" t="n">
         <v>30</v>
@@ -4105,12 +4114,12 @@
         <v>37</v>
       </c>
       <c r="M51" s="7" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="N51" s="12"/>
       <c r="O51" s="12"/>
       <c r="P51" s="7" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="Q51" s="7" t="s">
         <v>37</v>
@@ -4120,54 +4129,54 @@
       </c>
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="23"/>
-      <c r="B52" s="23"/>
-      <c r="C52" s="24" t="s">
-        <v>276</v>
-      </c>
-      <c r="D52" s="23"/>
-      <c r="E52" s="23"/>
-      <c r="F52" s="23"/>
-      <c r="G52" s="23"/>
-      <c r="H52" s="23"/>
-      <c r="I52" s="25" t="n">
+      <c r="A52" s="29"/>
+      <c r="B52" s="29"/>
+      <c r="C52" s="30" t="s">
+        <v>269</v>
+      </c>
+      <c r="D52" s="29"/>
+      <c r="E52" s="29"/>
+      <c r="F52" s="29"/>
+      <c r="G52" s="29"/>
+      <c r="H52" s="29"/>
+      <c r="I52" s="31" t="n">
         <f aca="false">SUMIFS($I$5:$I$51,$F$5:$F$51,"SHIP")</f>
         <v>80</v>
       </c>
-      <c r="J52" s="23"/>
-      <c r="K52" s="23"/>
-      <c r="L52" s="23"/>
-      <c r="M52" s="23"/>
-      <c r="N52" s="23"/>
-      <c r="O52" s="23"/>
-      <c r="P52" s="23"/>
-      <c r="Q52" s="23"/>
-      <c r="R52" s="23"/>
+      <c r="J52" s="29"/>
+      <c r="K52" s="29"/>
+      <c r="L52" s="29"/>
+      <c r="M52" s="29"/>
+      <c r="N52" s="29"/>
+      <c r="O52" s="29"/>
+      <c r="P52" s="29"/>
+      <c r="Q52" s="29"/>
+      <c r="R52" s="29"/>
     </row>
     <row r="53" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="26"/>
-      <c r="B53" s="26"/>
-      <c r="C53" s="27" t="s">
-        <v>277</v>
-      </c>
-      <c r="D53" s="26"/>
-      <c r="E53" s="26"/>
-      <c r="F53" s="26"/>
-      <c r="G53" s="26"/>
-      <c r="H53" s="26"/>
-      <c r="I53" s="28" t="n">
+      <c r="A53" s="32"/>
+      <c r="B53" s="32"/>
+      <c r="C53" s="33" t="s">
+        <v>270</v>
+      </c>
+      <c r="D53" s="32"/>
+      <c r="E53" s="32"/>
+      <c r="F53" s="32"/>
+      <c r="G53" s="32"/>
+      <c r="H53" s="32"/>
+      <c r="I53" s="34" t="n">
         <f aca="false">I27+I35+I42+I52</f>
-        <v>485.89</v>
-      </c>
-      <c r="J53" s="26"/>
-      <c r="K53" s="26"/>
-      <c r="L53" s="26"/>
-      <c r="M53" s="26"/>
-      <c r="N53" s="26"/>
-      <c r="O53" s="26"/>
-      <c r="P53" s="26"/>
-      <c r="Q53" s="26"/>
-      <c r="R53" s="26"/>
+        <v>487.87</v>
+      </c>
+      <c r="J53" s="32"/>
+      <c r="K53" s="32"/>
+      <c r="L53" s="32"/>
+      <c r="M53" s="32"/>
+      <c r="N53" s="32"/>
+      <c r="O53" s="32"/>
+      <c r="P53" s="32"/>
+      <c r="Q53" s="32"/>
+      <c r="R53" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -4223,196 +4232,196 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>279</v>
-      </c>
-      <c r="B3" s="29" t="n">
+        <v>272</v>
+      </c>
+      <c r="B3" s="35" t="n">
         <v>380</v>
       </c>
-      <c r="C3" s="30" t="s">
-        <v>280</v>
+      <c r="C3" s="36" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="31" t="s">
-        <v>281</v>
-      </c>
-      <c r="B5" s="32" t="n">
+      <c r="A5" s="37" t="s">
+        <v>274</v>
+      </c>
+      <c r="B5" s="38" t="n">
         <f aca="false">SUMIFS(BOM!$I$5:$I$53,BOM!$F$5:$F$53,"P1")</f>
-        <v>133.65</v>
-      </c>
-      <c r="C5" s="31" t="s">
-        <v>282</v>
+        <v>135.63</v>
+      </c>
+      <c r="C5" s="37" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="31" t="s">
-        <v>283</v>
-      </c>
-      <c r="B6" s="32" t="n">
+      <c r="A6" s="37" t="s">
+        <v>276</v>
+      </c>
+      <c r="B6" s="38" t="n">
         <f aca="false">SUMIFS(BOM!$I$5:$I$53,BOM!$F$5:$F$53,"PCB")</f>
         <v>72.95</v>
       </c>
-      <c r="C6" s="31" t="s">
-        <v>284</v>
+      <c r="C6" s="37" t="s">
+        <v>277</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="31" t="s">
-        <v>285</v>
-      </c>
-      <c r="B7" s="32" t="n">
+      <c r="A7" s="37" t="s">
+        <v>278</v>
+      </c>
+      <c r="B7" s="38" t="n">
         <f aca="false">SUMIFS(BOM!$I$5:$I$53,BOM!$F$5:$F$53,"P2")</f>
         <v>199.29</v>
       </c>
-      <c r="C7" s="31" t="s">
-        <v>286</v>
+      <c r="C7" s="37" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="31" t="s">
-        <v>287</v>
-      </c>
-      <c r="B8" s="32" t="n">
+      <c r="A8" s="37" t="s">
+        <v>280</v>
+      </c>
+      <c r="B8" s="38" t="n">
         <f aca="false">SUMIFS(BOM!$I$5:$I$53,BOM!$F$5:$F$53,"SHIP")</f>
         <v>80</v>
       </c>
-      <c r="C8" s="31" t="s">
-        <v>288</v>
+      <c r="C8" s="37" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="31" t="s">
-        <v>289</v>
-      </c>
-      <c r="B9" s="32" t="n">
+      <c r="A9" s="37" t="s">
+        <v>282</v>
+      </c>
+      <c r="B9" s="38" t="n">
         <f aca="false">SUMIFS(BOM!$I$5:$I$53,BOM!$F$5:$F$53,"P3")</f>
         <v>0</v>
       </c>
-      <c r="C9" s="31" t="s">
-        <v>290</v>
+      <c r="C9" s="37" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="33" t="s">
-        <v>291</v>
-      </c>
-      <c r="B10" s="34" t="n">
+      <c r="A10" s="39" t="s">
+        <v>284</v>
+      </c>
+      <c r="B10" s="40" t="n">
         <f aca="false">SUM(B5:B9)</f>
-        <v>485.89</v>
+        <v>487.87</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="33" t="s">
-        <v>292</v>
-      </c>
-      <c r="B11" s="35" t="n">
+      <c r="A11" s="39" t="s">
+        <v>285</v>
+      </c>
+      <c r="B11" s="41" t="n">
         <f aca="false">B3-B10</f>
-        <v>-105.89</v>
-      </c>
-      <c r="C11" s="30" t="s">
-        <v>293</v>
+        <v>-107.87</v>
+      </c>
+      <c r="C11" s="36" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="31" t="s">
-        <v>294</v>
-      </c>
-      <c r="B13" s="32" t="n">
+      <c r="A13" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="B13" s="38" t="n">
         <f aca="false">SUMIFS(BOM!$H$5:$H$53,BOM!$F$5:$F$53,"P3")</f>
         <v>57.94</v>
       </c>
-      <c r="C13" s="30" t="s">
-        <v>295</v>
+      <c r="C13" s="36" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="31" t="s">
-        <v>220</v>
-      </c>
-      <c r="B14" s="32" t="n">
+      <c r="A14" s="37" t="s">
+        <v>213</v>
+      </c>
+      <c r="B14" s="38" t="n">
         <f aca="false">SUMIFS(BOM!$H$5:$H$53,BOM!$C$5:$C$53,"*Coral*")</f>
         <v>135</v>
       </c>
-      <c r="C14" s="30" t="s">
+      <c r="C14" s="36" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="39" t="s">
+        <v>290</v>
+      </c>
+      <c r="B16" s="40" t="n">
+        <f aca="false">B10</f>
+        <v>487.87</v>
+      </c>
+      <c r="C16" s="36" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="39" t="s">
+        <v>292</v>
+      </c>
+      <c r="B17" s="40" t="n">
+        <f aca="false">B10+B13+B14</f>
+        <v>680.81</v>
+      </c>
+      <c r="C17" s="36" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="37" t="s">
+        <v>294</v>
+      </c>
+      <c r="B19" s="37" t="n">
+        <f aca="false">COUNTIFS(BOM!$E$5:$E$53,"&gt;0",BOM!$G$5:$G$53,"Estimate")+COUNTIFS(BOM!$E$5:$E$53,"&gt;0",BOM!$H$5:$H$53,"")</f>
+        <v>6</v>
+      </c>
+      <c r="C19" s="36" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="37" t="s">
         <v>296</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="33" t="s">
+      <c r="B20" s="37" t="n">
+        <f aca="false">COUNTIFS(BOM!$E$5:$E$53,"&gt;0",BOM!$G$5:$G$53,"Verified")+COUNTIFS(BOM!$E$5:$E$53,"&gt;0",BOM!$G$5:$G$53,"Received")</f>
+        <v>8</v>
+      </c>
+      <c r="C20" s="36" t="s">
         <v>297</v>
       </c>
-      <c r="B16" s="34" t="n">
-        <f aca="false">B10</f>
-        <v>485.89</v>
-      </c>
-      <c r="C16" s="30" t="s">
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="39" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="33" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="37" t="s">
         <v>299</v>
       </c>
-      <c r="B17" s="34" t="n">
-        <f aca="false">B10+B13+B14</f>
-        <v>678.83</v>
-      </c>
-      <c r="C17" s="30" t="s">
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="37" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="31" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="37" t="s">
         <v>301</v>
       </c>
-      <c r="B19" s="31" t="n">
-        <f aca="false">COUNTIFS(BOM!$E$5:$E$53,"&gt;0",BOM!$G$5:$G$53,"Estimate")+COUNTIFS(BOM!$E$5:$E$53,"&gt;0",BOM!$H$5:$H$53,"")</f>
-        <v>8</v>
-      </c>
-      <c r="C19" s="30" t="s">
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="37" t="s">
         <v>302</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="31" t="s">
-        <v>303</v>
-      </c>
-      <c r="B20" s="31" t="n">
-        <f aca="false">COUNTIFS(BOM!$E$5:$E$53,"&gt;0",BOM!$G$5:$G$53,"Verified")</f>
-        <v>6</v>
-      </c>
-      <c r="C20" s="30" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="33" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="31" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="31" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="31" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="31" t="s">
-        <v>309</v>
       </c>
     </row>
   </sheetData>
@@ -4431,7 +4440,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
@@ -4439,81 +4448,89 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="31"/>
+      <c r="B1" s="37"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="39" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="37" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="39" t="s">
+        <v>304</v>
+      </c>
+      <c r="B3" s="37" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="39" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="37" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="39" t="s">
+        <v>133</v>
+      </c>
+      <c r="B5" s="37" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="39" t="s">
+        <v>308</v>
+      </c>
+      <c r="B6" s="37" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="39" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="33" t="s">
-        <v>74</v>
-      </c>
-      <c r="B3" s="31" t="s">
+      <c r="B7" s="37" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="33" t="s">
-        <v>92</v>
-      </c>
-      <c r="B4" s="31" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="39" t="s">
         <v>312</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="33" t="s">
+      <c r="B8" s="37" t="s">
         <v>313</v>
       </c>
-      <c r="B5" s="31" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="39" t="s">
         <v>314</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="33" t="s">
+      <c r="B9" s="37" t="s">
         <v>315</v>
       </c>
-      <c r="B6" s="31" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="39" t="s">
         <v>316</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="33" t="s">
+      <c r="B10" s="37" t="s">
         <v>317</v>
       </c>
-      <c r="B7" s="31" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="39" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="33" t="s">
+      <c r="B11" s="37" t="s">
         <v>319</v>
-      </c>
-      <c r="B8" s="31" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="33" t="s">
-        <v>321</v>
-      </c>
-      <c r="B9" s="31" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="33" t="s">
-        <v>323</v>
-      </c>
-      <c r="B10" s="31" t="s">
-        <v>324</v>
       </c>
     </row>
   </sheetData>
@@ -4546,17 +4563,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -4568,19 +4585,19 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>12</v>
@@ -4589,162 +4606,162 @@
         <v>13</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="C6" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="36" t="n">
+      <c r="D6" s="42" t="n">
         <v>39.99</v>
       </c>
-      <c r="E6" s="37" t="n">
+      <c r="E6" s="43" t="n">
         <f aca="false">C6*D6</f>
         <v>79.98</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>13</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="36" t="n">
+      <c r="D7" s="42" t="n">
         <v>19.99</v>
       </c>
-      <c r="E7" s="37" t="n">
+      <c r="E7" s="43" t="n">
         <f aca="false">C7*D7</f>
         <v>19.99</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G7" s="11" t="s">
         <v>13</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>333</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>338</v>
       </c>
       <c r="C8" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="36" t="n">
+      <c r="D8" s="42" t="n">
         <v>6.69</v>
       </c>
-      <c r="E8" s="37" t="n">
+      <c r="E8" s="43" t="n">
         <f aca="false">C8*D8</f>
         <v>6.69</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G8" s="11" t="s">
         <v>13</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="C9" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="36" t="n">
-        <v>5</v>
-      </c>
-      <c r="E9" s="37" t="n">
+      <c r="D9" s="42" t="n">
+        <v>5.99</v>
+      </c>
+      <c r="E9" s="43" t="n">
         <f aca="false">C9*D9</f>
-        <v>5</v>
+        <v>5.99</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>341</v>
+        <v>46</v>
       </c>
       <c r="G9" s="11" t="s">
         <v>13</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>342</v>
+        <v>336</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
       <c r="C10" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="36" t="n">
-        <v>6</v>
-      </c>
-      <c r="E10" s="37" t="n">
+      <c r="D10" s="42" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="E10" s="43" t="n">
         <f aca="false">C10*D10</f>
-        <v>6</v>
+        <v>6.99</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>341</v>
+        <v>46</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>13</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="23"/>
-      <c r="B11" s="24" t="s">
-        <v>345</v>
-      </c>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="25" t="n">
+      <c r="A11" s="29"/>
+      <c r="B11" s="30" t="s">
+        <v>339</v>
+      </c>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="31" t="n">
         <f aca="false">SUM(E6:E10)</f>
-        <v>117.66</v>
-      </c>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="23"/>
+        <v>119.64</v>
+      </c>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -4756,19 +4773,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>12</v>
@@ -4777,23 +4794,23 @@
         <v>13</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="C15" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D15" s="36" t="n">
+      <c r="D15" s="42" t="n">
         <v>0.99</v>
       </c>
-      <c r="E15" s="37" t="n">
+      <c r="E15" s="43" t="n">
         <f aca="false">C15*D15</f>
         <v>0.99</v>
       </c>
@@ -4804,27 +4821,27 @@
         <v>13</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23"/>
-      <c r="B16" s="24" t="s">
-        <v>349</v>
-      </c>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="25" t="n">
+      <c r="A16" s="29"/>
+      <c r="B16" s="30" t="s">
+        <v>344</v>
+      </c>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="31" t="n">
         <f aca="false">SUM(E15:E15)</f>
         <v>0.99</v>
       </c>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
+      <c r="F16" s="29"/>
+      <c r="G16" s="29"/>
+      <c r="H16" s="29"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -4836,19 +4853,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>12</v>
@@ -4857,48 +4874,48 @@
         <v>13</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="C20" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D20" s="36" t="n">
+      <c r="D20" s="42" t="n">
         <v>15</v>
       </c>
-      <c r="E20" s="37" t="n">
+      <c r="E20" s="43" t="n">
         <f aca="false">C20*D20</f>
         <v>15</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="G20" s="7"/>
       <c r="H20" s="7" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="C21" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="36" t="n">
+      <c r="D21" s="42" t="n">
         <v>20.13</v>
       </c>
-      <c r="E21" s="37" t="n">
+      <c r="E21" s="43" t="n">
         <f aca="false">C21*D21</f>
         <v>20.13</v>
       </c>
@@ -4909,54 +4926,54 @@
         <v>13</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="C22" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="36" t="n">
+      <c r="D22" s="42" t="n">
         <v>11.99</v>
       </c>
-      <c r="E22" s="37" t="n">
+      <c r="E22" s="43" t="n">
         <f aca="false">C22*D22</f>
         <v>11.99</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G22" s="11" t="s">
         <v>13</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="23"/>
-      <c r="B23" s="24" t="s">
-        <v>357</v>
-      </c>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="25" t="n">
+      <c r="A23" s="29"/>
+      <c r="B23" s="30" t="s">
+        <v>352</v>
+      </c>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="31" t="n">
         <f aca="false">SUM(E20:E22)</f>
         <v>47.12</v>
       </c>
-      <c r="F23" s="23"/>
-      <c r="G23" s="23"/>
-      <c r="H23" s="23"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="29"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="2" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
     </row>
   </sheetData>
@@ -5002,182 +5019,182 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="38" t="s">
-        <v>359</v>
+      <c r="A1" s="44" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="39" t="s">
-        <v>360</v>
+      <c r="A2" s="45" t="s">
+        <v>355</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="40" t="s">
-        <v>361</v>
+      <c r="A3" s="46" t="s">
+        <v>356</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="F6" s="14"/>
     </row>
     <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="F7" s="14"/>
     </row>
     <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="E9" s="14"/>
       <c r="F9" s="14"/>
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="F10" s="14"/>
     </row>
     <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>2</v>
       </c>
       <c r="D11" s="14" t="s">
+        <v>374</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>372</v>
+      </c>
+      <c r="F11" s="14"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="47"/>
+      <c r="B14" s="48" t="s">
+        <v>375</v>
+      </c>
+      <c r="C14" s="47"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="47"/>
+      <c r="F14" s="47"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="37" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="37" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="37" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="37" t="s">
         <v>379</v>
       </c>
-      <c r="E11" s="14" t="s">
-        <v>377</v>
-      </c>
-      <c r="F11" s="14"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="41"/>
-      <c r="B14" s="42" t="s">
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="37" t="s">
         <v>380</v>
       </c>
-      <c r="C14" s="41"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="41"/>
-      <c r="F14" s="41"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="31" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="37" t="s">
         <v>381</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="31" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="31" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="31" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="31" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="31" t="s">
-        <v>386</v>
       </c>
     </row>
   </sheetData>

</xml_diff>